<commit_message>
Add US dollar equivalents to monetary values: Australia, Nigeria, New Zealand
Each local-currency amount in the profile and summary now carries its US$
equivalent in parentheses, computed by scripts/fx.py from data/fx_rates.json
(22 October 2026 reference rates). Documents, PDFs and packages rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChEN58PbdXFZmwUoBZYBRb
</commit_message>
<xml_diff>
--- a/deliverables/Australia/Partnerships_Tracker.xlsx
+++ b/deliverables/Australia/Partnerships_Tracker.xlsx
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tracker" displayName="Tracker" ref="A1:L122" headerRowCount="1">
-  <autoFilter ref="A1:L122"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tracker" displayName="Tracker" ref="A1:L165" headerRowCount="1">
+  <autoFilter ref="A1:L165"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Status"/>
     <tableColumn id="2" name="Country"/>
@@ -558,7 +558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scope: partnerships that are active, or ended or last active within the past five years. Last checked 2026-10-20.</t>
+          <t>Scope: partnerships that are active, or ended or last active within the past five years. Last checked 2026-10-21.</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$122,A5)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$165,A5)</f>
         <v/>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$122,A6)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$165,A6)</f>
         <v/>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$122,A7)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$165,A7)</f>
         <v/>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7732,6 +7732,2496 @@
       <c r="L122" s="14" t="inlineStr">
         <is>
           <t>The Edge Malaysia, 2024-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B123" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C123" s="13" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Bloomberg School of Public Health, Center for Indigenous Health)</t>
+        </is>
+      </c>
+      <c r="D123" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E123" s="12" t="inlineStr">
+        <is>
+          <t>University of Otago, Te Rōpū Rangahau Hauora a Eru Pōmare (Eru Pōmare Māori Health Research Centre)</t>
+        </is>
+      </c>
+      <c r="F123" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G123" s="12" t="inlineStr">
+        <is>
+          <t>The Johns Hopkins Center for Indigenous Health runs the SPIRIT collective, a five year program funded by the LEGO Foundation that adapts its Family Spirit home visiting model and builds Indigenous playspaces. Its lead partner in New Zealand is the Eru Pōmare Māori Health Research Centre at the University of Otago, working with three Māori community sites.</t>
+        </is>
+      </c>
+      <c r="H123" s="12" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="I123" s="12" t="inlineStr"/>
+      <c r="J123" s="12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="K123" s="12" t="inlineStr">
+        <is>
+          <t>JHCIH won the LEGO Foundation Build a World of Play Challenge in December 2022 and funding began in 2023. A JHCIH Q&amp;A published 21 January 2026 says the program is past its halfway point and names the University of Otago's Eru Pōmare centre as lead partner in Aotearoa, with partners meeting in Alice Springs in August 2024. The program page lists its status as Active.</t>
+        </is>
+      </c>
+      <c r="L123" s="14" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Center for Indigenous Health, 2026-01-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B124" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C124" s="13" t="inlineStr">
+        <is>
+          <t>Icon Oncology Group (Icon Group)</t>
+        </is>
+      </c>
+      <c r="D124" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E124" s="12" t="inlineStr">
+        <is>
+          <t>Bowen Icon Cancer Centre (joint venture with Evolution Healthcare, Bowen Hospital)</t>
+        </is>
+      </c>
+      <c r="F124" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G124" s="12" t="inlineStr">
+        <is>
+          <t>Icon, Australia's largest dedicated cancer care provider, co-owns and runs the Bowen Icon Cancer Centre in Wellington as a joint venture with Evolution Healthcare. The centre offers private chemotherapy, haematology and, since 2019, radiation therapy.</t>
+        </is>
+      </c>
+      <c r="H124" s="12" t="inlineStr">
+        <is>
+          <t>2017-07</t>
+        </is>
+      </c>
+      <c r="I124" s="12" t="inlineStr"/>
+      <c r="J124" s="12" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="K124" s="12" t="inlineStr">
+        <is>
+          <t>Newshub reported the Prime Minister opening the centre in July 2017. Icon's current group pages (copyright 2026, and mentioning its 2024 Pharmaxo acquisition) still describe Bowen Icon Cancer Centre as a joint venture with Evolution Healthcare, and the centre's own site is live under Icon branding. None of these pages carries a dated news item on the joint venture after 2017, so Active rests on current corporate pages rather than a dated release. Icon's 4 February 2025 news item says it introduced clinical trials at Bowen Icon Cancer Centre.</t>
+        </is>
+      </c>
+      <c r="L124" s="14" t="inlineStr">
+        <is>
+          <t>Icon Oncology Group, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B125" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C125" s="13" t="inlineStr">
+        <is>
+          <t>National University of Singapore and National University Health System</t>
+        </is>
+      </c>
+      <c r="D125" s="12" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="E125" s="12" t="inlineStr">
+        <is>
+          <t>Liggins Institute, University of Auckland</t>
+        </is>
+      </c>
+      <c r="F125" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G125" s="12" t="inlineStr">
+        <is>
+          <t>The Liggins Institute has formal agreements with the National University of Singapore and works with NUS and National University Hospital in the EpiGen consortium. Their joint NiPPeR trial and child follow-up study enrolled families in Auckland, Singapore and Southampton.</t>
+        </is>
+      </c>
+      <c r="H125" s="12" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="I125" s="12" t="inlineStr"/>
+      <c r="J125" s="12" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="K125" s="12" t="inlineStr">
+        <is>
+          <t>The Liggins Institute's partnerships page cites formal agreements with NUS and the Singapore Institute for Clinical Sciences. The NiPPeR Child study (NCT05934422) names NUS, NUHS and National University Hospital as collaborators and Shiao-Yng Chan of NUS as a principal investigator alongside Auckland. It completed in August 2025, and the record was updated in November 2025. The NiPPeR Child follow-up ran from June 2023 to its completion on 14 August 2025.</t>
+        </is>
+      </c>
+      <c r="L125" s="14" t="inlineStr">
+        <is>
+          <t>University of Auckland</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B126" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C126" s="13" t="inlineStr">
+        <is>
+          <t>UCLPartners</t>
+        </is>
+      </c>
+      <c r="D126" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E126" s="12" t="inlineStr">
+        <is>
+          <t>Health New Zealand Te Whatu Ora (HealthX programme)</t>
+        </is>
+      </c>
+      <c r="F126" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G126" s="12" t="inlineStr">
+        <is>
+          <t>Health New Zealand's HealthX programme signed an agreement with UCLPartners, the London academic health science partnership of NHS organisations and universities. UCLPartners advises on testing and scaling digital and AI tools such as emergency department AI scribes.</t>
+        </is>
+      </c>
+      <c r="H126" s="12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I126" s="12" t="inlineStr"/>
+      <c r="J126" s="12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="K126" s="12" t="inlineStr">
+        <is>
+          <t>A Health NZ sector update republished by HiNZ on 8 July 2026 announces the agreement, quotes Health NZ chief executive Dale Bramley and UCLPartners chief executive Chris Laing, and says UCLPartners horizon scanning already informed the AI scribe rollout.</t>
+        </is>
+      </c>
+      <c r="L126" s="14" t="inlineStr">
+        <is>
+          <t>HiNZ (eHealthNews.nz), 2026-07-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B127" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C127" s="13" t="inlineStr">
+        <is>
+          <t>Universitas Indonesia (Faculty of Public Health)</t>
+        </is>
+      </c>
+      <c r="D127" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="E127" s="12" t="inlineStr">
+        <is>
+          <t>University of Otago (Faculty of Medicine)</t>
+        </is>
+      </c>
+      <c r="F127" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G127" s="12" t="inlineStr">
+        <is>
+          <t>Universitas Indonesia's Faculty of Public Health and Otago's Faculty of Medicine signed an implementation agreement for a joint Master of Public Health, with study split between Jakarta and Otago. It builds on a 2024 university MoU.</t>
+        </is>
+      </c>
+      <c r="H127" s="12" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I127" s="12" t="inlineStr"/>
+      <c r="J127" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="K127" s="12" t="inlineStr">
+        <is>
+          <t>An FPH UI release dated 31 October 2025 reports that Otago's Associate Dean of International Health Sciences signed the Agreement of Implementation on a 23 to 24 October 2025 visit, extending MoU No. 56/MOU/R/UI/2024.</t>
+        </is>
+      </c>
+      <c r="L127" s="14" t="inlineStr">
+        <is>
+          <t>Universitas Indonesia, 2025-11-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B128" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C128" s="13" t="inlineStr">
+        <is>
+          <t>University of Southampton (MRC Lifecourse Epidemiology Centre, EpiGen Global Research Consortium)</t>
+        </is>
+      </c>
+      <c r="D128" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E128" s="12" t="inlineStr">
+        <is>
+          <t>Liggins Institute, University of Auckland</t>
+        </is>
+      </c>
+      <c r="F128" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G128" s="12" t="inlineStr">
+        <is>
+          <t>Southampton and the University of Auckland's Liggins Institute are founding partners of the EpiGen Global Research Consortium, with Singapore partners. Together they run the NiPPeR preconception nutrition trial and its child follow-up study.</t>
+        </is>
+      </c>
+      <c r="H128" s="12" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="I128" s="12" t="inlineStr"/>
+      <c r="J128" s="12" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="K128" s="12" t="inlineStr">
+        <is>
+          <t>The Liggins Institute lists itself as a foundation partner of EpiGen, established 2006, with two Southampton units. The NiPPeR Child follow-up study (NCT05934422), sponsored by Southampton with Auckland as a site and Wayne Cutfield as a principal investigator, ran from June 2023 to August 2025, and its registry record was updated in November 2025. The NiPPeR Child follow-up ran from June 2023 to its completion on 14 August 2025.</t>
+        </is>
+      </c>
+      <c r="L128" s="14" t="inlineStr">
+        <is>
+          <t>University of Auckland</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B129" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C129" s="13" t="inlineStr">
+        <is>
+          <t>University of Wollongong (Graduate School of Medicine)</t>
+        </is>
+      </c>
+      <c r="D129" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E129" s="12" t="inlineStr">
+        <is>
+          <t>University of Waikato (New Zealand Graduate School of Medicine)</t>
+        </is>
+      </c>
+      <c r="F129" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G129" s="12" t="inlineStr">
+        <is>
+          <t>Wollongong and Waikato signed a memorandum of understanding under which Wollongong's rural medical education staff help design the curriculum of Waikato's new graduate entry medical school. The school focuses on primary care, rural health and equity.</t>
+        </is>
+      </c>
+      <c r="H129" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="I129" s="12" t="inlineStr"/>
+      <c r="J129" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="K129" s="12" t="inlineStr">
+        <is>
+          <t>A University of Wollongong release dated 17 October 2025 announces the MoU signing by Vice-Chancellors Max Lu and Neil Quigley, with quotes from Waikato's Pro Vice-Chancellor Health.</t>
+        </is>
+      </c>
+      <c r="L129" s="14" t="inlineStr">
+        <is>
+          <t>University of Wollongong, 2025-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B130" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C130" s="13" t="inlineStr">
+        <is>
+          <t>West Visayas State University</t>
+        </is>
+      </c>
+      <c r="D130" s="12" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="E130" s="12" t="inlineStr">
+        <is>
+          <t>University of Otago</t>
+        </is>
+      </c>
+      <c r="F130" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G130" s="12" t="inlineStr">
+        <is>
+          <t>West Visayas State University and Otago signed a memorandum of understanding covering joint research in digital health and medicine, faculty and student exchange, and co-development of digital health tools.</t>
+        </is>
+      </c>
+      <c r="H130" s="12" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="I130" s="12" t="inlineStr"/>
+      <c r="J130" s="12" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="K130" s="12" t="inlineStr">
+        <is>
+          <t>A WVSU release reports the MoU was signed on 27 June 2025 in Dunedin by WVSU President Joselito Villaruz and Otago Vice-Chancellor Grant Robertson during a CHED higher education mission. No Otago-side release was found.</t>
+        </is>
+      </c>
+      <c r="L130" s="14" t="inlineStr">
+        <is>
+          <t>West Visayas State University, 2025-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B131" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C131" s="13" t="inlineStr">
+        <is>
+          <t>Sanford Health (Sanford World Clinic)</t>
+        </is>
+      </c>
+      <c r="D131" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E131" s="12" t="inlineStr">
+        <is>
+          <t>Omni Health (OmniHealth) primary care network</t>
+        </is>
+      </c>
+      <c r="F131" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G131" s="12" t="inlineStr">
+        <is>
+          <t>Sanford World Clinic and Omni Health opened a general practice clinic in central Auckland in early 2018 and Sanford has since invested in and helped run Omni Health's national primary care network. The network now has about 22 medical centres in 21 towns, and Sanford recruits doctors for it.</t>
+        </is>
+      </c>
+      <c r="H131" s="12" t="inlineStr">
+        <is>
+          <t>2018-01</t>
+        </is>
+      </c>
+      <c r="I131" s="12" t="inlineStr"/>
+      <c r="J131" s="12" t="inlineStr">
+        <is>
+          <t>2021-05</t>
+        </is>
+      </c>
+      <c r="K131" s="12" t="inlineStr">
+        <is>
+          <t>A May 2021 SiouxFalls.Business report says Sanford helped build a $30 million network of clinics with Omni Health through multiple investments, with a Sanford executive acting as its COO from Sioux Falls. Sanford's current World Clinic page says it has collaborated with Omni Health since 2018. Sanford World Clinic's recruiting page on PracticeMatch lists Omni Health physician openings posted 6 October 2025. The October 2025 recruitment listing could not be re-verified; Sanford's current page says in the present tense that it has collaborated with Omni Health since 2018 but carries no date.</t>
+        </is>
+      </c>
+      <c r="L131" s="14" t="inlineStr">
+        <is>
+          <t>Sanford Health</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B132" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C132" s="13" t="inlineStr">
+        <is>
+          <t>Children's Cancer Institute and Sydney Children's Hospital, Randwick (Zero Childhood Cancer Program)</t>
+        </is>
+      </c>
+      <c r="D132" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E132" s="12" t="inlineStr">
+        <is>
+          <t>Starship Children's Hospital and Christchurch Hospital (Health New Zealand)</t>
+        </is>
+      </c>
+      <c r="F132" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G132" s="12" t="inlineStr">
+        <is>
+          <t>The ZERO precision medicine program, led by Children's Cancer Institute and Sydney Children's Hospital Randwick, opened to New Zealand children in 2024. Starship's tumours are sent for genomic analysis that guides treatment, and Christchurch was listed as a second site.</t>
+        </is>
+      </c>
+      <c r="H132" s="12" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="I132" s="12" t="inlineStr"/>
+      <c r="J132" s="12" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="K132" s="12" t="inlineStr">
+        <is>
+          <t>ANZCHOG, the study sponsor, announced on 19 August 2024 that ZERO2 opened at Starship on 17 July 2024. The ZERO2 registry record (NCT05504772, last updated July 2024) lists Starship as recruiting and Christchurch as not yet recruiting. Children's Cancer Institute's undated program page says both New Zealand sites opened in 2024. No dated evidence from October 2024 or later was found.</t>
+        </is>
+      </c>
+      <c r="L132" s="14" t="inlineStr">
+        <is>
+          <t>Australian and New Zealand Children's Haematology/Oncology Group, 2024-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B133" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C133" s="13" t="inlineStr">
+        <is>
+          <t>Children's Hospital of Zhejiang University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D133" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E133" s="12" t="inlineStr">
+        <is>
+          <t>NZ-China Non-Communicable Diseases Research Collaboration Centre (University of Otago)</t>
+        </is>
+      </c>
+      <c r="F133" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G133" s="12" t="inlineStr">
+        <is>
+          <t>The Children's Hospital of Zhejiang University signed a 2017 memorandum of understanding with the Otago-hosted NZ-China NCD Research Collaboration Centre on childhood obesity and diabetes research. Its vice president presented at the centre's 2022 forum.</t>
+        </is>
+      </c>
+      <c r="H133" s="12" t="inlineStr">
+        <is>
+          <t>2017-10</t>
+        </is>
+      </c>
+      <c r="I133" s="12" t="inlineStr"/>
+      <c r="J133" s="12" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="K133" s="12" t="inlineStr">
+        <is>
+          <t>The centre reported the October 2017 MoU signing. Its report on the 5 to 6 July 2022 forum cites a presentation by the hospital's vice president Jun-Fen Fu on obesity and diabetes in children. Nothing later was found. Later evidence is forum participation only (a virtual 2022 forum); the MoU dates from 2017.</t>
+        </is>
+      </c>
+      <c r="L133" s="14" t="inlineStr">
+        <is>
+          <t>NZ-China NCD CRCC, 2017-11-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B134" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C134" s="13" t="inlineStr">
+        <is>
+          <t>Fiji National University (College of Medicine, Nursing and Health Sciences)</t>
+        </is>
+      </c>
+      <c r="D134" s="12" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="E134" s="12" t="inlineStr">
+        <is>
+          <t>University of Auckland</t>
+        </is>
+      </c>
+      <c r="F134" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G134" s="12" t="inlineStr">
+        <is>
+          <t>Fiji National University and the University of Auckland signed a memorandum of understanding, driven by FNU's medical college and Auckland's paediatrics department, covering staff capacity building, exchanges and joint research.</t>
+        </is>
+      </c>
+      <c r="H134" s="12" t="inlineStr">
+        <is>
+          <t>2022-05</t>
+        </is>
+      </c>
+      <c r="I134" s="12" t="inlineStr"/>
+      <c r="J134" s="12" t="inlineStr">
+        <is>
+          <t>2022-05</t>
+        </is>
+      </c>
+      <c r="K134" s="12" t="inlineStr">
+        <is>
+          <t>An FNU press release dated 9 May 2022 reports the MoU signing, attended by Auckland paediatrics Associate Professor Stephen Howie. No later activity was found.</t>
+        </is>
+      </c>
+      <c r="L134" s="14" t="inlineStr">
+        <is>
+          <t>Fiji National University, 2022-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B135" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C135" s="13" t="inlineStr">
+        <is>
+          <t>Huashan Hospital (Fudan University)</t>
+        </is>
+      </c>
+      <c r="D135" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E135" s="12" t="inlineStr">
+        <is>
+          <t>NZ-China Non-Communicable Diseases Research Collaboration Centre (University of Otago)</t>
+        </is>
+      </c>
+      <c r="F135" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G135" s="12" t="inlineStr">
+        <is>
+          <t>Huashan Hospital signed a 2017 memorandum of understanding with the Otago-hosted NZ-China NCD Research Collaboration Centre for joint research on brain and other non-communicable diseases. Its researchers took part in the centre's 2022 forum.</t>
+        </is>
+      </c>
+      <c r="H135" s="12" t="inlineStr">
+        <is>
+          <t>2017-10</t>
+        </is>
+      </c>
+      <c r="I135" s="12" t="inlineStr"/>
+      <c r="J135" s="12" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="K135" s="12" t="inlineStr">
+        <is>
+          <t>The centre reported the October 2017 signing of four MoUs including Huashan. Its report on the 3rd NZ-China NCD forum, held 5 to 6 July 2022, cites a Huashan Hospital presentation on AI digital monitoring. Nothing later was found. Later evidence is forum participation only (a virtual 2022 forum); the MoU dates from 2017.</t>
+        </is>
+      </c>
+      <c r="L135" s="14" t="inlineStr">
+        <is>
+          <t>NZ-China NCD CRCC, 2017-11-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B136" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C136" s="13" t="inlineStr">
+        <is>
+          <t>Shanghai Ninth People's Hospital (Shanghai Jiao Tong University School of Medicine)</t>
+        </is>
+      </c>
+      <c r="D136" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E136" s="12" t="inlineStr">
+        <is>
+          <t>University of Otago Faculty of Dentistry</t>
+        </is>
+      </c>
+      <c r="F136" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G136" s="12" t="inlineStr">
+        <is>
+          <t>Shanghai Ninth People's Hospital and Otago's Faculty of Dentistry signed a memorandum of understanding and opened the Shanghai-New Zealand Joint Laboratory of Dentistry for craniofacial research.</t>
+        </is>
+      </c>
+      <c r="H136" s="12" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="I136" s="12" t="inlineStr"/>
+      <c r="J136" s="12" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="K136" s="12" t="inlineStr">
+        <is>
+          <t>A Shanghai Jiao Tong University School of Medicine release dated 28 November 2023 reports the signing on 27 November 2023 by hospital president Wu Hao and Otago dental dean Paul Cooper. No later activity was found.</t>
+        </is>
+      </c>
+      <c r="L136" s="14" t="inlineStr">
+        <is>
+          <t>Shanghai Jiao Tong University School of Medicine, 2023-11-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="16" t="inlineStr">
+        <is>
+          <t>Ended</t>
+        </is>
+      </c>
+      <c r="B137" s="12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C137" s="13" t="inlineStr">
+        <is>
+          <t>Healthe Care Australia (then a subsidiary of Luye Medical Group)</t>
+        </is>
+      </c>
+      <c r="D137" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E137" s="12" t="inlineStr">
+        <is>
+          <t>Boulcott Hospital (Pulse Health NZ)</t>
+        </is>
+      </c>
+      <c r="F137" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G137" s="12" t="inlineStr">
+        <is>
+          <t>Healthe Care, an Australian private hospital operator, owned Pulse Health NZ and through it ran Boulcott Hospital in Lower Hutt. It sold Pulse Health NZ to a Pacific Equity Partners vehicle in late 2021, and Boulcott's operations passed to Rangatira Investments in March 2022.</t>
+        </is>
+      </c>
+      <c r="H137" s="12" t="inlineStr">
+        <is>
+          <t>2017-05</t>
+        </is>
+      </c>
+      <c r="I137" s="12" t="inlineStr">
+        <is>
+          <t>2021-11</t>
+        </is>
+      </c>
+      <c r="J137" s="12" t="inlineStr">
+        <is>
+          <t>2022-03</t>
+        </is>
+      </c>
+      <c r="K137" s="12" t="inlineStr">
+        <is>
+          <t>Healthe Care acquired ASX-listed Pulse Health, Boulcott's operator, in May 2017. The Commerce Commission on 17 November 2021 cleared Pacific 2021 Bidco to buy 100% of Pulse Health NZ from Healthe Care, on condition that Boulcott be sold. NBR reported on 2 March 2022 that Rangatira Investments had bought Boulcott's operations. The end month is the clearance date; completion fell between November 2021 and March 2022.</t>
+        </is>
+      </c>
+      <c r="L137" s="14" t="inlineStr">
+        <is>
+          <t>Commerce Commission New Zealand, 2021-11-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B138" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C138" s="13" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Johns Hopkins Hospital)</t>
+        </is>
+      </c>
+      <c r="D138" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E138" s="12" t="inlineStr">
+        <is>
+          <t>Afe Babalola University (ABUAD)</t>
+        </is>
+      </c>
+      <c r="F138" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G138" s="12" t="inlineStr">
+        <is>
+          <t>Tripartite agreement with the Little by Little Foundation letting high performing ABUAD medical students do part of their fifth year clinical electives at Johns Hopkins Hospital.</t>
+        </is>
+      </c>
+      <c r="H138" s="12" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="I138" s="12" t="inlineStr"/>
+      <c r="J138" s="12" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="K138" s="12" t="inlineStr">
+        <is>
+          <t>ABUAD notice dated 17 January 2023 reports the signing on 10 January 2023. No later evidence of placements found in 2024 to 2026 searches. ABUAD's 5 February 2025 release on its seventh induction ceremony describes the six-week Johns Hopkins Hospital electives as ongoing.</t>
+        </is>
+      </c>
+      <c r="L138" s="14" t="inlineStr">
+        <is>
+          <t>Afe Babalola University, 2023-01-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B139" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C139" s="13" t="inlineStr">
+        <is>
+          <t>Mayo Clinic (Mayo Clinic Global Consulting)</t>
+        </is>
+      </c>
+      <c r="D139" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E139" s="12" t="inlineStr">
+        <is>
+          <t>Iwosan Investments Limited (Iwosan Lagoon Hospitals and Lagos Medipark Hospital)</t>
+        </is>
+      </c>
+      <c r="F139" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G139" s="12" t="inlineStr">
+        <is>
+          <t>Iwosan Investments, owner of the Iwosan Lagoon Hospitals group, engaged Mayo Clinic Global Consulting for strategic advice on organisation and clinical practice. The work starts with Iwosan Lagoon Hospitals and the planned Lagos Medipark Hospital.</t>
+        </is>
+      </c>
+      <c r="H139" s="12" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="I139" s="12" t="inlineStr"/>
+      <c r="J139" s="12" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="K139" s="12" t="inlineStr">
+        <is>
+          <t>Iwosan's announcement was syndicated on 17 April 2025 (The Sun) and carried by BusinessDay and BrandIconImage. No page on Mayo's own newsroom was found, so confirmation rests on the Nigerian company's release. No end date or contract term is stated.</t>
+        </is>
+      </c>
+      <c r="L139" s="14" t="inlineStr">
+        <is>
+          <t>The Sun Nigeria, 2025-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C140" s="13" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="D140" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E140" s="12" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH) and College of Medicine, University of Lagos</t>
+        </is>
+      </c>
+      <c r="F140" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G140" s="12" t="inlineStr">
+        <is>
+          <t>LUTH and the University of Lagos College of Medicine serve as research and training hubs of the MSK founded ARGO consortium. They take part in joint cancer studies, including a colorectal cancer immunotherapy trial.</t>
+        </is>
+      </c>
+      <c r="H140" s="12" t="inlineStr"/>
+      <c r="I140" s="12" t="inlineStr"/>
+      <c r="J140" s="12" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="K140" s="12" t="inlineStr">
+        <is>
+          <t>MSK's 2025 GCRT Update names OAUTHC and the College of Medicine, University of Lagos/LUTH as ARGO's research and training hubs. MSK's press page describes the colorectal immunotherapy trial with OAUTHC, LUTH and Medserve. Start year not stated on a dated page.</t>
+        </is>
+      </c>
+      <c r="L140" s="14" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B141" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C141" s="13" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="D141" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E141" s="12" t="inlineStr">
+        <is>
+          <t>Obafemi Awolowo University Teaching Hospitals Complex (OAUTHC)</t>
+        </is>
+      </c>
+      <c r="F141" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G141" s="12" t="inlineStr">
+        <is>
+          <t>MSK's Global Cancer Research and Training program partners with OAUTHC, home of the African Research Group for Oncology (ARGO), an NCI recognised consortium founded in 2013. The work covers cancer research, trials and training for Nigerian clinicians.</t>
+        </is>
+      </c>
+      <c r="H141" s="12" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="I141" s="12" t="inlineStr"/>
+      <c r="J141" s="12" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="K141" s="12" t="inlineStr">
+        <is>
+          <t>MSK's 2025 GCRT Update reports the annual ARGO symposium held at Ile-Ife in September 2025 and a colorectal immunotherapy trial run with OAUTHC. MSK's program page dates the partnership to the 2009 training of OAUTHC surgeon Isaac Alatise; start year is that visit, ARGO itself dates to 2013.</t>
+        </is>
+      </c>
+      <c r="L141" s="14" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B142" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C142" s="13" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="D142" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E142" s="12" t="inlineStr">
+        <is>
+          <t>Abubakar Tafawa Balewa University Teaching Hospital (ATBUTH)</t>
+        </is>
+      </c>
+      <c r="F142" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G142" s="12" t="inlineStr">
+        <is>
+          <t>ATBUTH signed a Medical Institution Membership Agreement and joined the St. Jude Global Alliance, a care and training network for childhood cancer. Membership gives access to mentorship, shared treatment protocols and training.</t>
+        </is>
+      </c>
+      <c r="H142" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="I142" s="12" t="inlineStr"/>
+      <c r="J142" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="K142" s="12" t="inlineStr">
+        <is>
+          <t>Leadership newspaper published the hospital's statement on 26 October 2025 (signing described as the day before). Not confirmed on St. Jude's own site.</t>
+        </is>
+      </c>
+      <c r="L142" s="14" t="inlineStr">
+        <is>
+          <t>Leadership Newspapers, 2025-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B143" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C143" s="13" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="D143" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E143" s="12" t="inlineStr">
+        <is>
+          <t>The Dorcas Cancer Foundation (TDCF)</t>
+        </is>
+      </c>
+      <c r="F143" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G143" s="12" t="inlineStr">
+        <is>
+          <t>TDCF joined the St. Jude Global Alliance as the first Nigerian non profit member, to improve paediatric cancer outcomes in Nigeria and sub Saharan Africa. TDCF runs a paediatric radiation oncology training course.</t>
+        </is>
+      </c>
+      <c r="H143" s="12" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="I143" s="12" t="inlineStr"/>
+      <c r="J143" s="12" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="K143" s="12" t="inlineStr">
+        <is>
+          <t>ThisDay and BusinessDay reported the admission on 17 December 2024. The Nigerian party is a non profit, not a hospital, and the tie is an alliance membership; flag for the verifier. Not confirmed on St. Jude's site. Caveat: the Nigerian party is a cancer foundation working with pediatric oncology units, not a hospital.</t>
+        </is>
+      </c>
+      <c r="L143" s="14" t="inlineStr">
+        <is>
+          <t>ThisDay, 2024-12-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B144" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C144" s="13" t="inlineStr">
+        <is>
+          <t>University of Illinois Chicago (UIC School of Public Health)</t>
+        </is>
+      </c>
+      <c r="D144" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E144" s="12" t="inlineStr">
+        <is>
+          <t>Lagos State University (LASU)</t>
+        </is>
+      </c>
+      <c r="F144" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G144" s="12" t="inlineStr">
+        <is>
+          <t>Framework agreement signed 28 July 2026 for academic collaboration, joint research and student and faculty exchange, focused on urban health, emergency preparedness and AI-enabled public health tools.</t>
+        </is>
+      </c>
+      <c r="H144" s="12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I144" s="12" t="inlineStr"/>
+      <c r="J144" s="12" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="K144" s="12" t="inlineStr">
+        <is>
+          <t>UIC School of Public Health news, 4 August 2026, reports the memorandum signed on 28 July 2026 in Chicago by LASU's Vice Chancellor and UIC representatives. A university to university agreement with no hospital named.</t>
+        </is>
+      </c>
+      <c r="L144" s="14" t="inlineStr">
+        <is>
+          <t>UIC School of Public Health, 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B145" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C145" s="13" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine (Institute of Human Virology)</t>
+        </is>
+      </c>
+      <c r="D145" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E145" s="12" t="inlineStr">
+        <is>
+          <t>Institute of Human Virology Nigeria (IHVN)</t>
+        </is>
+      </c>
+      <c r="F145" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G145" s="12" t="inlineStr">
+        <is>
+          <t>IHVN is the Nigerian affiliate of the Maryland Institute of Human Virology, delivering HIV, TB and cancer care, training and research. It opened a multi campus site in Abuja in 2023.</t>
+        </is>
+      </c>
+      <c r="H145" s="12" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="I145" s="12" t="inlineStr"/>
+      <c r="J145" s="12" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="K145" s="12" t="inlineStr">
+        <is>
+          <t>University of Maryland news from June 2023 reports the Abuja campus launch with UMB leadership present. No dated evidence from October 2024 onward found. IHVN is an NGO affiliate, not a hospital; flag for the verifier. NIH RePORTER shows Fogarty training grant D43TW012280 awarded to IHVN for FY2026 (budget start 1 February 2026), co-led with the UMSOM Institute of Human Virology. Caveat: IHVN is the Institute's Nigerian NGO affiliate, not a hospital.</t>
+        </is>
+      </c>
+      <c r="L145" s="14" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine, 2023-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B146" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C146" s="13" t="inlineStr">
+        <is>
+          <t>University of Miami (Sylvester Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="D146" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E146" s="12" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University Teaching Hospital (ABUTH)</t>
+        </is>
+      </c>
+      <c r="F146" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G146" s="12" t="inlineStr">
+        <is>
+          <t>ABUTH is a recruiting site in a University of Miami led trial of niraparib maintenance therapy for ovarian cancer in women of African ancestry. The tie began with a Miami delegation visit to ABUTH in 2023.</t>
+        </is>
+      </c>
+      <c r="H146" s="12" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="I146" s="12" t="inlineStr"/>
+      <c r="J146" s="12" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="K146" s="12" t="inlineStr">
+        <is>
+          <t>ClinicalTrials.gov NCT06412120 lists ABUTH Zaria as recruiting, study start 28 July 2026, record updated 5 August 2026, Miami investigators Schlumbrecht and George. ABUTH's August 2023 news item reports the planning visit (page not retrievable; seen in search results only).</t>
+        </is>
+      </c>
+      <c r="L146" s="14" t="inlineStr">
+        <is>
+          <t>US National Library of Medicine, 2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B147" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C147" s="13" t="inlineStr">
+        <is>
+          <t>University of Virginia Health System</t>
+        </is>
+      </c>
+      <c r="D147" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E147" s="12" t="inlineStr">
+        <is>
+          <t>Federal Medical Centre Umuahia</t>
+        </is>
+      </c>
+      <c r="F147" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G147" s="12" t="inlineStr">
+        <is>
+          <t>UVA nephrology supports the kidney transplant programme at FMC Umuahia through mentorship, coordinator training and joint research under the ISN and TTS Sister Transplant Centers Program. The pair reached Level B in 2026.</t>
+        </is>
+      </c>
+      <c r="H147" s="12" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I147" s="12" t="inlineStr"/>
+      <c r="J147" s="12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="K147" s="12" t="inlineStr">
+        <is>
+          <t>UVA Medicine in Motion news, 13 May 2026, reports the move from Level C to Level B, shorter post transplant stays (14 to 8 days), four trained coordinators and eight joint publications in the first two years, which puts the start near 2024.</t>
+        </is>
+      </c>
+      <c r="L147" s="14" t="inlineStr">
+        <is>
+          <t>UVA Medicine in Motion, 2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C148" s="13" t="inlineStr">
+        <is>
+          <t>Vanderbilt University Medical Center (Vanderbilt Institute for Global Health)</t>
+        </is>
+      </c>
+      <c r="D148" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E148" s="12" t="inlineStr">
+        <is>
+          <t>Aminu Kano Teaching Hospital and Bayero University Kano</t>
+        </is>
+      </c>
+      <c r="F148" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G148" s="12" t="inlineStr">
+        <is>
+          <t>Long running research and training partnership, now in its second Fogarty funded phase (V-BRCH 2), building Nigerian capacity for clinical research on HIV and related chronic diseases. Related programmes cover child neurology and research administration.</t>
+        </is>
+      </c>
+      <c r="H148" s="12" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="I148" s="12" t="inlineStr"/>
+      <c r="J148" s="12" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="K148" s="12" t="inlineStr">
+        <is>
+          <t>Fogarty grant D43TW011544 lists Aminu Kano Teaching Hospital as principal institution with award years 2020 to 2029, and Vanderbilt's V-BRCH page describes V-BRCH 2 as a continuation. Both pages are undated, so last evidence reflects page content as read on 16 October 2026; flag for the verifier. Start year is the 2020 award; the AKTH tie is older. Fogarty grant D43TW011544 was renewed in 2025 with Aminu Kano Teaching Hospital as grantee; the FY2026 award notice is dated 18 December 2025 (NIH RePORTER).</t>
+        </is>
+      </c>
+      <c r="L148" s="14" t="inlineStr">
+        <is>
+          <t>US National Institutes of Health</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B149" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C149" s="13" t="inlineStr">
+        <is>
+          <t>Virginia Commonwealth University (VCU Massey Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="D149" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E149" s="12" t="inlineStr">
+        <is>
+          <t>National Hospital Abuja</t>
+        </is>
+      </c>
+      <c r="F149" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G149" s="12" t="inlineStr">
+        <is>
+          <t>Two year memorandum of understanding between the National Hospital and VCU Massey Comprehensive Cancer Center to build cancer research capacity. Focus areas are clinical trials, training of new scientists and moving research into patient care.</t>
+        </is>
+      </c>
+      <c r="H149" s="12" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="I149" s="12" t="inlineStr"/>
+      <c r="J149" s="12" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="K149" s="12" t="inlineStr">
+        <is>
+          <t>News Agency of Nigeria and Nairametrics reported the signing on 1 July 2025 by Prof Muhammad Mahmud and Dr Robert Winn, saying it was signed on a Tuesday (24 June or 1 July 2025). Term is two years, so it runs to mid 2027.</t>
+        </is>
+      </c>
+      <c r="L149" s="14" t="inlineStr">
+        <is>
+          <t>Nairametrics, 2025-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B150" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C150" s="13" t="inlineStr">
+        <is>
+          <t>Evercare Group (owned at its 2021 launch by the TPG-managed Evercare Health Fund)</t>
+        </is>
+      </c>
+      <c r="D150" s="12" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="E150" s="12" t="inlineStr">
+        <is>
+          <t>Evercare Hospital Lekki</t>
+        </is>
+      </c>
+      <c r="F150" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G150" s="12" t="inlineStr">
+        <is>
+          <t>Evercare Group owns and operates Evercare Hospital Lekki, a 165-bed tertiary hospital in Lagos that opened in February 2021, as part of its network of hospitals in Africa and South Asia.</t>
+        </is>
+      </c>
+      <c r="H150" s="12" t="inlineStr">
+        <is>
+          <t>2021-03</t>
+        </is>
+      </c>
+      <c r="I150" s="12" t="inlineStr"/>
+      <c r="J150" s="12" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="K150" s="12" t="inlineStr">
+        <is>
+          <t>ThisDay, 10 October 2024, describes Evercare Hospital Lekki as part of the Evercare Group, which operates in Kenya and Pakistan as well as Nigeria, announcing new cochlear implant surgery. TPG's release and a 2021 report document the group's ownership and the February 2021 opening. A 2026 LinkedIn post suggests continued operation but was not verified. Ownership is as of the 2021 launch; no later ownership confirmation was found.</t>
+        </is>
+      </c>
+      <c r="L150" s="14" t="inlineStr">
+        <is>
+          <t>ThisDay, 2024-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B151" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C151" s="13" t="inlineStr">
+        <is>
+          <t>King's College Hospital NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="D151" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E151" s="12" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="F151" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G151" s="12" t="inlineStr">
+        <is>
+          <t>King's is the appointed Clinical Partner of the AMCE, supporting clinical protocols, governance, service set-up, recruitment and training for the 170-bed specialist hospital in Abuja. Clinical services were commissioned in June 2025.</t>
+        </is>
+      </c>
+      <c r="H151" s="12" t="inlineStr">
+        <is>
+          <t>2021-06</t>
+        </is>
+      </c>
+      <c r="I151" s="12" t="inlineStr"/>
+      <c r="J151" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K151" s="12" t="inlineStr">
+        <is>
+          <t>Afreximbank announced on 3 June 2021 that it had signed an agreement appointing King's College Hospital as Clinical Partner. Nairametrics reports the AMCE was commissioned on 5 June 2025 with Vice President Shettima praising the AMCE and King's partnership. Brand Spur (19 September 2026) describes the centre as developed with King's College Hospital and now commissioned.</t>
+        </is>
+      </c>
+      <c r="L151" s="14" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (amce.net), 2021-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B152" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C152" s="13" t="inlineStr">
+        <is>
+          <t>King's College London</t>
+        </is>
+      </c>
+      <c r="D152" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E152" s="12" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="F152" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G152" s="12" t="inlineStr">
+        <is>
+          <t>King's College London and Afreximbank agreed to plan a medical and nursing school at the AMCE in Abuja, drawing on King's healthcare education expertise. A further terms of agreement was signed in June 2025.</t>
+        </is>
+      </c>
+      <c r="H152" s="12" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="I152" s="12" t="inlineStr"/>
+      <c r="J152" s="12" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="K152" s="12" t="inlineStr">
+        <is>
+          <t>King's news release of 28 November 2023 reports the memorandum of agreement signed on 24 November 2023 for a scoping study of the school. Nairametrics reports a terms of agreement between Afreximbank and King's College London on the school was signed at the AMCE commissioning on 5 June 2025.</t>
+        </is>
+      </c>
+      <c r="L152" s="14" t="inlineStr">
+        <is>
+          <t>King's College London, 2023-11-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B153" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C153" s="13" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine</t>
+        </is>
+      </c>
+      <c r="D153" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E153" s="12" t="inlineStr">
+        <is>
+          <t>National Postgraduate Medical College of Nigeria (with Wellbeing Foundation Africa)</t>
+        </is>
+      </c>
+      <c r="F153" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G153" s="12" t="inlineStr">
+        <is>
+          <t>LSTM leads Advanced Obstetrics and Surgical Skills training for obstetrics and gynaecology examiners and residents of the National Postgraduate Medical College, with centres of excellence in Lagos and Abuja and later sites in Port Harcourt and Gombe. It is funded by the UK Global Health Workforce Programme.</t>
+        </is>
+      </c>
+      <c r="H153" s="12" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="I153" s="12" t="inlineStr"/>
+      <c r="J153" s="12" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="K153" s="12" t="inlineStr">
+        <is>
+          <t>LSTM reports the course began on 6 May 2024 at the college's centre of excellence at LUTH. The Wellbeing Foundation Africa reported on 12 February 2025 that 225 doctors had been trained, and on 22 May 2025 that training had expanded to the University of Port Harcourt Teaching Hospital. LSTM's May 2024 release names the site as 'Lagos State University Teaching Hospital (LUTH)', which is ambiguous; WBFA reported 225 examiners and 120 residents trained by May 2025.</t>
+        </is>
+      </c>
+      <c r="L153" s="14" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine, 2024-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B154" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C154" s="13" t="inlineStr">
+        <is>
+          <t>Manipal Hospitals</t>
+        </is>
+      </c>
+      <c r="D154" s="12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E154" s="12" t="inlineStr">
+        <is>
+          <t>Afe Babalola University Multi-System Hospital</t>
+        </is>
+      </c>
+      <c r="F154" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G154" s="12" t="inlineStr">
+        <is>
+          <t>Afe Babalola University Multi-System Hospital and Manipal Hospitals signed an MoU to expand capacity, deepen specialist training, improve clinical exchange and support advanced surgical care.</t>
+        </is>
+      </c>
+      <c r="H154" s="12" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="I154" s="12" t="inlineStr"/>
+      <c r="J154" s="12" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="K154" s="12" t="inlineStr">
+        <is>
+          <t>News Agency of Nigeria, 26 June 2026, reports the MoU announced at a press briefing by the hospital's chief medical director, with Dr Rajit Sood speaking for Manipal and the university's Vice-Chancellor present.</t>
+        </is>
+      </c>
+      <c r="L154" s="14" t="inlineStr">
+        <is>
+          <t>News Agency of Nigeria, 2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B155" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C155" s="13" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="D155" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E155" s="12" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="F155" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G155" s="12" t="inlineStr">
+        <is>
+          <t>The Christie, through Christie International, is the oncology partner to King's College Hospital in advising the AMCE, supporting oncology staff recruitment, education and quality assurance. It continues to support the oncology service after opening.</t>
+        </is>
+      </c>
+      <c r="H155" s="12" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="I155" s="12" t="inlineStr"/>
+      <c r="J155" s="12" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="K155" s="12" t="inlineStr">
+        <is>
+          <t>The Christie's news story of 25 October 2024 reports an AMCE delegation visit to Manchester and says its advice, which began in 2021, would continue into operations. The Christie's project page, as indexed in search, states that clinical services were commissioned on 5 June 2025 with Christie International's head attending.</t>
+        </is>
+      </c>
+      <c r="L155" s="14" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust, 2024-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B156" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C156" s="13" t="inlineStr">
+        <is>
+          <t>The Royal Marsden NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="D156" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E156" s="12" t="inlineStr">
+        <is>
+          <t>Marcelle Ruth Cancer Centre &amp; Specialist Hospital</t>
+        </is>
+      </c>
+      <c r="F156" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G156" s="12" t="inlineStr">
+        <is>
+          <t>The two cancer centres signed a strategic partnership covering clinical expertise, research, professional development and training, aimed at keeping cancer care in Nigeria and West Africa.</t>
+        </is>
+      </c>
+      <c r="H156" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="I156" s="12" t="inlineStr"/>
+      <c r="J156" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K156" s="12" t="inlineStr">
+        <is>
+          <t>BusinessDay reported on 24 September 2026 that Marcelle Ruth had entered a strategic partnership with The Royal Marsden. Search results also show the agreement described as an MoU on a Royal Marsden Private Care LinkedIn post; no Royal Marsden press release was found.</t>
+        </is>
+      </c>
+      <c r="L156" s="14" t="inlineStr">
+        <is>
+          <t>BusinessDay, 2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B157" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C157" s="13" t="inlineStr">
+        <is>
+          <t>University of Birmingham</t>
+        </is>
+      </c>
+      <c r="D157" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E157" s="12" t="inlineStr">
+        <is>
+          <t>University of Lagos (with Lagos University Teaching Hospital)</t>
+        </is>
+      </c>
+      <c r="F157" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G157" s="12" t="inlineStr">
+        <is>
+          <t>The University of Lagos and the University of Birmingham signed a memorandum on transnational education covering student and staff exchange and curriculum development. It builds on more than a decade of global surgery collaboration that introduced a master's programme in surgery at LUTH.</t>
+        </is>
+      </c>
+      <c r="H157" s="12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="I157" s="12" t="inlineStr"/>
+      <c r="J157" s="12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="K157" s="12" t="inlineStr">
+        <is>
+          <t>Vanguard, 29 January 2026, reports the MoU signed at UNILAG's Senate Chamber, witnessed by the Minister of Education; UNILAG's Vice Chancellor cites the Birmingham global surgery work and the LUTH master's in surgery. Birmingham described the MoU as a statement of intent. Not yet confirmed on Birmingham's newsroom.</t>
+        </is>
+      </c>
+      <c r="L157" s="14" t="inlineStr">
+        <is>
+          <t>Vanguard, 29 January 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B158" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C158" s="13" t="inlineStr">
+        <is>
+          <t>University of Glasgow</t>
+        </is>
+      </c>
+      <c r="D158" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E158" s="12" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University</t>
+        </is>
+      </c>
+      <c r="F158" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G158" s="12" t="inlineStr">
+        <is>
+          <t>A university-level MoU provides a framework for joint research programmes, postgraduate co-supervision and academic exchange on global health challenges, coordinated by the School of Infection and Immunity. A university-wide MoU; no teaching-hospital or clinical component is named.</t>
+        </is>
+      </c>
+      <c r="H158" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="I158" s="12" t="inlineStr"/>
+      <c r="J158" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="K158" s="12" t="inlineStr">
+        <is>
+          <t>The University of Glasgow news item of 12 May 2026 reports the MoU signed during a visit on 28 and 29 April 2026, following an exploratory visit in December 2025. The MoU is university-wide and not limited to the teaching hospital.</t>
+        </is>
+      </c>
+      <c r="L158" s="14" t="inlineStr">
+        <is>
+          <t>University of Glasgow, 2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B159" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C159" s="13" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine</t>
+        </is>
+      </c>
+      <c r="D159" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E159" s="12" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH)</t>
+        </is>
+      </c>
+      <c r="F159" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G159" s="12" t="inlineStr">
+        <is>
+          <t>The University of Maryland School of Medicine and LUTH announced a chronic disease collaboration in August 2024, initially for four to five years with a stated ten-year ambition.</t>
+        </is>
+      </c>
+      <c r="H159" s="12" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="I159" s="12" t="inlineStr"/>
+      <c r="J159" s="12" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="K159" s="12" t="inlineStr">
+        <is>
+          <t>Nairametrics (19 August 2024) and LUTH report a partnership planned over ten years, following a visit by Dean Mark Gladwin. No signed text or later 2024 to 2026 update found, so it falls just before the Active cutoff.</t>
+        </is>
+      </c>
+      <c r="L159" s="14" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital, 2024-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B160" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C160" s="13" t="inlineStr">
+        <is>
+          <t>University of Virginia Health System</t>
+        </is>
+      </c>
+      <c r="D160" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E160" s="12" t="inlineStr">
+        <is>
+          <t>Federal Medical Centre Owo</t>
+        </is>
+      </c>
+      <c r="F160" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G160" s="12" t="inlineStr">
+        <is>
+          <t>UVA's nephrology division built a partnership with FMC Owo covering research and career development programmes, with the International Society of Nephrology, and donated textbooks.</t>
+        </is>
+      </c>
+      <c r="H160" s="12" t="inlineStr"/>
+      <c r="I160" s="12" t="inlineStr"/>
+      <c r="J160" s="12" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="K160" s="12" t="inlineStr">
+        <is>
+          <t>UVA news item describes a textbook donation on 6 January 2023. No later dated evidence found, and the work may now sit inside the FMC Umuahia programme.</t>
+        </is>
+      </c>
+      <c r="L160" s="14" t="inlineStr">
+        <is>
+          <t>UVA Medicine in Motion, 2023-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B161" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C161" s="13" t="inlineStr">
+        <is>
+          <t>Yale School of Medicine (Department of Psychiatry)</t>
+        </is>
+      </c>
+      <c r="D161" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E161" s="12" t="inlineStr">
+        <is>
+          <t>Imo State University Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="F161" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G161" s="12" t="inlineStr">
+        <is>
+          <t>Yale's HAPPINESS Project, run with the Imo State teaching hospital, trains primary care workers to treat mental, neurological and substance use disorders, with telemedicine specialist support. It has begun integrating mental health into HIV clinics.</t>
+        </is>
+      </c>
+      <c r="H161" s="12" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="I161" s="12" t="inlineStr"/>
+      <c r="J161" s="12" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="K161" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria Health Watch, 6 September 2023, reports over 100 workers trained; Yale's programme page is undated. No dated evidence from October 2024 onward found. The teaching hospital is in Orlu, Imo State.</t>
+        </is>
+      </c>
+      <c r="L161" s="14" t="inlineStr">
+        <is>
+          <t>Nigeria Health Watch, 2023-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B162" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C162" s="13" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="D162" s="12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E162" s="12" t="inlineStr">
+        <is>
+          <t>Duchess International Hospital (Reddington Hospital Group)</t>
+        </is>
+      </c>
+      <c r="F162" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G162" s="12" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals supports the operation and management of the 100-bed Duchess International Hospital in Ikeja, Lagos, to strengthen efficiency and clinical quality. The arrangement was announced when the hospital launched in October 2021.</t>
+        </is>
+      </c>
+      <c r="H162" s="12" t="inlineStr">
+        <is>
+          <t>2021-10</t>
+        </is>
+      </c>
+      <c r="I162" s="12" t="inlineStr"/>
+      <c r="J162" s="12" t="inlineStr">
+        <is>
+          <t>2021-11</t>
+        </is>
+      </c>
+      <c r="K162" s="12" t="inlineStr">
+        <is>
+          <t>ThisDay (11 November 2021) and New Telegraph report that operation and management of the Duchess are supported by Apollo Hospitals, India. No dated confirmation from October 2024 onward was found; the hospital's 2024 and 2025 award releases do not mention Apollo.</t>
+        </is>
+      </c>
+      <c r="L162" s="14" t="inlineStr">
+        <is>
+          <t>ThisDay, 11 November 2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B163" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C163" s="13" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="D163" s="12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E163" s="12" t="inlineStr">
+        <is>
+          <t>State House Clinic</t>
+        </is>
+      </c>
+      <c r="F163" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G163" s="12" t="inlineStr">
+        <is>
+          <t>Apollo doctors visit the State House Clinic to give free consultations and lectures, and clinic staff have been sent to Apollo in India for up to six weeks of training at no charge.</t>
+        </is>
+      </c>
+      <c r="H163" s="12" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="I163" s="12" t="inlineStr"/>
+      <c r="J163" s="12" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="K163" s="12" t="inlineStr">
+        <is>
+          <t>Blueprint, 29 July 2022, quotes the clinic's medical director describing a collaboration of almost six to seven years and a visiting Apollo team in Abuja. Start year is approximate, back-calculated from that quote. No later dated activity was found; a March 2024 ThisDay report records only Apollo's stated intent to partner with Nigerian hospitals.</t>
+        </is>
+      </c>
+      <c r="L163" s="14" t="inlineStr">
+        <is>
+          <t>Blueprint, 2022-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B164" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="inlineStr">
+        <is>
+          <t>Memorial Hospitals Group</t>
+        </is>
+      </c>
+      <c r="D164" s="12" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="E164" s="12" t="inlineStr">
+        <is>
+          <t>Kasi Healthcare</t>
+        </is>
+      </c>
+      <c r="F164" s="12" t="inlineStr">
+        <is>
+          <t>Telehealth and second opinion</t>
+        </is>
+      </c>
+      <c r="G164" s="12" t="inlineStr">
+        <is>
+          <t>Memorial specialists provide second opinions and specialist screenings, with monthly visiting specialists and training courses for Nigerian providers at Kasi's Lagos airport clinic, linked to referral of patients to Turkey. Close to a patient-referral arrangement.</t>
+        </is>
+      </c>
+      <c r="H164" s="12" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="I164" s="12" t="inlineStr"/>
+      <c r="J164" s="12" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="K164" s="12" t="inlineStr">
+        <is>
+          <t>BusinessDay, 27 September 2024, reports the partnership announced with Memorial's country executive. No later dated activity was found.</t>
+        </is>
+      </c>
+      <c r="L164" s="14" t="inlineStr">
+        <is>
+          <t>BusinessDay, 2024-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B165" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C165" s="13" t="inlineStr">
+        <is>
+          <t>Peking University People's Hospital (named variously in press as People's University Hospital, Beijing)</t>
+        </is>
+      </c>
+      <c r="D165" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E165" s="12" t="inlineStr">
+        <is>
+          <t>University of Abuja Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="F165" s="12" t="inlineStr">
+        <is>
+          <t>Government agreement</t>
+        </is>
+      </c>
+      <c r="G165" s="12" t="inlineStr">
+        <is>
+          <t>A China-Nigeria government letter of intent names these two hospitals as the pioneer project for hospital cooperation under the 2021 FOCAC health programmes, covering knowledge sharing and research.</t>
+        </is>
+      </c>
+      <c r="H165" s="12" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="I165" s="12" t="inlineStr"/>
+      <c r="J165" s="12" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="K165" s="12" t="inlineStr">
+        <is>
+          <t>Within Nigeria and the University of Abuja Teaching Hospital website report the letter of intent signed in Abuja by the Chinese Ambassador and Nigeria's Health Minister in August 2022. No follow-up activity was found. The Chinese hospital's name varies between sources and is inferred.</t>
+        </is>
+      </c>
+      <c r="L165" s="14" t="inlineStr">
+        <is>
+          <t>Within Nigeria, 2022-08-20</t>
         </is>
       </c>
     </row>
@@ -7858,10 +10348,53 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L165" r:id="rId164"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId122"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId165"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7872,7 +10405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E244"/>
+  <dimension ref="A1:E328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -14455,6 +16988,2230 @@
       <c r="E244" s="5" t="inlineStr">
         <is>
           <t>https://theedgemalaysia.com/node/725855</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Bloomberg School of Public Health, Center for Indigenous Health)</t>
+        </is>
+      </c>
+      <c r="B245" s="5" t="inlineStr">
+        <is>
+          <t>University of Otago, Te Rōpū Rangahau Hauora a Eru Pōmare (Eru Pōmare Māori Health Research Centre)</t>
+        </is>
+      </c>
+      <c r="C245" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Center for Indigenous Health SPIRIT Program Q&amp;A: A Global Collaboration Rooted In Indigenous Play</t>
+        </is>
+      </c>
+      <c r="D245" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="E245" s="5" t="inlineStr">
+        <is>
+          <t>https://cih.jhu.edu/spirit-program-qa</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Bloomberg School of Public Health, Center for Indigenous Health)</t>
+        </is>
+      </c>
+      <c r="B246" s="5" t="inlineStr">
+        <is>
+          <t>University of Otago, Te Rōpū Rangahau Hauora a Eru Pōmare (Eru Pōmare Māori Health Research Centre)</t>
+        </is>
+      </c>
+      <c r="C246" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Center for Indigenous Health SPIRIT</t>
+        </is>
+      </c>
+      <c r="D246" s="5" t="inlineStr"/>
+      <c r="E246" s="5" t="inlineStr">
+        <is>
+          <t>https://cih.jhu.edu/programs/spirit/</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Bloomberg School of Public Health, Center for Indigenous Health)</t>
+        </is>
+      </c>
+      <c r="B247" s="5" t="inlineStr">
+        <is>
+          <t>University of Otago, Te Rōpū Rangahau Hauora a Eru Pōmare (Eru Pōmare Māori Health Research Centre)</t>
+        </is>
+      </c>
+      <c r="C247" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University Bloomberg School announces expanded Center for Indigenous Health</t>
+        </is>
+      </c>
+      <c r="D247" s="5" t="inlineStr">
+        <is>
+          <t>2022-09-15</t>
+        </is>
+      </c>
+      <c r="E247" s="5" t="inlineStr">
+        <is>
+          <t>https://hub.jhu.edu/2022/09/15/center-for-indigenous-health-johns-hopkins/</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="5" t="inlineStr">
+        <is>
+          <t>Icon Oncology Group (Icon Group)</t>
+        </is>
+      </c>
+      <c r="B248" s="5" t="inlineStr">
+        <is>
+          <t>Bowen Icon Cancer Centre (joint venture with Evolution Healthcare, Bowen Hospital)</t>
+        </is>
+      </c>
+      <c r="C248" s="5" t="inlineStr">
+        <is>
+          <t>Icon Oncology Group About us</t>
+        </is>
+      </c>
+      <c r="D248" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E248" s="5" t="inlineStr">
+        <is>
+          <t>https://icongroup.global/about-us/</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="5" t="inlineStr">
+        <is>
+          <t>Icon Oncology Group (Icon Group)</t>
+        </is>
+      </c>
+      <c r="B249" s="5" t="inlineStr">
+        <is>
+          <t>Bowen Icon Cancer Centre (joint venture with Evolution Healthcare, Bowen Hospital)</t>
+        </is>
+      </c>
+      <c r="C249" s="5" t="inlineStr">
+        <is>
+          <t>Icon Oncology Group Cancer Services – New Zealand</t>
+        </is>
+      </c>
+      <c r="D249" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E249" s="5" t="inlineStr">
+        <is>
+          <t>https://icongroup.global/our-services/cancer-services-new-zealand/</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="5" t="inlineStr">
+        <is>
+          <t>Icon Oncology Group (Icon Group)</t>
+        </is>
+      </c>
+      <c r="B250" s="5" t="inlineStr">
+        <is>
+          <t>Bowen Icon Cancer Centre (joint venture with Evolution Healthcare, Bowen Hospital)</t>
+        </is>
+      </c>
+      <c r="C250" s="5" t="inlineStr">
+        <is>
+          <t>Newshub PM opens Wellington's first private cancer care facility</t>
+        </is>
+      </c>
+      <c r="D250" s="5" t="inlineStr">
+        <is>
+          <t>2017-07</t>
+        </is>
+      </c>
+      <c r="E250" s="5" t="inlineStr">
+        <is>
+          <t>https://www.newshub.co.nz/home/health/2017/07/pm-opens-wellington-s-first-private-cancer-care-facility.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="5" t="inlineStr">
+        <is>
+          <t>Icon Oncology Group (Icon Group)</t>
+        </is>
+      </c>
+      <c r="B251" s="5" t="inlineStr">
+        <is>
+          <t>Bowen Icon Cancer Centre (joint venture with Evolution Healthcare, Bowen Hospital)</t>
+        </is>
+      </c>
+      <c r="C251" s="5" t="inlineStr">
+        <is>
+          <t>Icon Writers United by Unique this World Cancer Day</t>
+        </is>
+      </c>
+      <c r="D251" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-04</t>
+        </is>
+      </c>
+      <c r="E251" s="5" t="inlineStr">
+        <is>
+          <t>https://icongroup.global/en/news/2025-02-04/world-cancer-day/</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="5" t="inlineStr">
+        <is>
+          <t>National University of Singapore and National University Health System</t>
+        </is>
+      </c>
+      <c r="B252" s="5" t="inlineStr">
+        <is>
+          <t>Liggins Institute, University of Auckland</t>
+        </is>
+      </c>
+      <c r="C252" s="5" t="inlineStr">
+        <is>
+          <t>Liggins Institute Research partnerships</t>
+        </is>
+      </c>
+      <c r="D252" s="5" t="inlineStr"/>
+      <c r="E252" s="5" t="inlineStr">
+        <is>
+          <t>https://www.auckland.ac.nz/en/liggins/in-the-community/scientists-researchers/research-partnerships.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="5" t="inlineStr">
+        <is>
+          <t>National University of Singapore and National University Health System</t>
+        </is>
+      </c>
+      <c r="B253" s="5" t="inlineStr">
+        <is>
+          <t>Liggins Institute, University of Auckland</t>
+        </is>
+      </c>
+      <c r="C253" s="5" t="inlineStr">
+        <is>
+          <t>University of Southampton NiPPeR Randomised Trial - Child Follow Up Study (NCT05934422)</t>
+        </is>
+      </c>
+      <c r="D253" s="5" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="E253" s="5" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT05934422</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="5" t="inlineStr">
+        <is>
+          <t>UCLPartners</t>
+        </is>
+      </c>
+      <c r="B254" s="5" t="inlineStr">
+        <is>
+          <t>Health New Zealand Te Whatu Ora (HealthX programme)</t>
+        </is>
+      </c>
+      <c r="C254" s="5" t="inlineStr">
+        <is>
+          <t>Health New Zealand Te Whatu Ora Health NZ international partnership strengthens approach to digital and AI innovation</t>
+        </is>
+      </c>
+      <c r="D254" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="E254" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hinz.org.nz/news/730824/Health-NZ-international-partnership-strengthens-digital-innovation.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Indonesia (Faculty of Public Health)</t>
+        </is>
+      </c>
+      <c r="B255" s="5" t="inlineStr">
+        <is>
+          <t>University of Otago (Faculty of Medicine)</t>
+        </is>
+      </c>
+      <c r="C255" s="5" t="inlineStr">
+        <is>
+          <t>Faculty of Public Health, Universitas Indonesia FPH UI and the University of Otago, New Zealand: joint Master of Public Health agreement</t>
+        </is>
+      </c>
+      <c r="D255" s="5" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
+        </is>
+      </c>
+      <c r="E255" s="5" t="inlineStr">
+        <is>
+          <t>https://fkm.ui.ac.id/?p=44053</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="5" t="inlineStr">
+        <is>
+          <t>University of Southampton (MRC Lifecourse Epidemiology Centre, EpiGen Global Research Consortium)</t>
+        </is>
+      </c>
+      <c r="B256" s="5" t="inlineStr">
+        <is>
+          <t>Liggins Institute, University of Auckland</t>
+        </is>
+      </c>
+      <c r="C256" s="5" t="inlineStr">
+        <is>
+          <t>Liggins Institute EpiGen Global Research Consortium</t>
+        </is>
+      </c>
+      <c r="D256" s="5" t="inlineStr"/>
+      <c r="E256" s="5" t="inlineStr">
+        <is>
+          <t>https://auckland.ac.nz/en/liggins/in-the-community/scientists-researchers/research-partnerships/epigen.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="5" t="inlineStr">
+        <is>
+          <t>University of Southampton (MRC Lifecourse Epidemiology Centre, EpiGen Global Research Consortium)</t>
+        </is>
+      </c>
+      <c r="B257" s="5" t="inlineStr">
+        <is>
+          <t>Liggins Institute, University of Auckland</t>
+        </is>
+      </c>
+      <c r="C257" s="5" t="inlineStr">
+        <is>
+          <t>University of Southampton NiPPeR Randomised Trial - Child Follow Up Study (NCT05934422)</t>
+        </is>
+      </c>
+      <c r="D257" s="5" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="E257" s="5" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT05934422</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="5" t="inlineStr">
+        <is>
+          <t>University of Wollongong (Graduate School of Medicine)</t>
+        </is>
+      </c>
+      <c r="B258" s="5" t="inlineStr">
+        <is>
+          <t>University of Waikato (New Zealand Graduate School of Medicine)</t>
+        </is>
+      </c>
+      <c r="C258" s="5" t="inlineStr">
+        <is>
+          <t>University of Wollongong Wollongong and Waikato partner to shape future of rural health in New Zealand</t>
+        </is>
+      </c>
+      <c r="D258" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="E258" s="5" t="inlineStr">
+        <is>
+          <t>https://www.uow.edu.au/media/2025/wollongong-and-waikato-partner-to-shape-future-of-rural-health-in-new-zealand.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="5" t="inlineStr">
+        <is>
+          <t>University of Wollongong (Graduate School of Medicine)</t>
+        </is>
+      </c>
+      <c r="B259" s="5" t="inlineStr">
+        <is>
+          <t>University of Waikato (New Zealand Graduate School of Medicine)</t>
+        </is>
+      </c>
+      <c r="C259" s="5" t="inlineStr">
+        <is>
+          <t>University of Waikato Waikato to work with regional health education experts to shape med school curriculum</t>
+        </is>
+      </c>
+      <c r="D259" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="E259" s="5" t="inlineStr">
+        <is>
+          <t>https://www.waikato.ac.nz/news-events/news/waikato-wollongong-mou/</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="5" t="inlineStr">
+        <is>
+          <t>West Visayas State University</t>
+        </is>
+      </c>
+      <c r="B260" s="5" t="inlineStr">
+        <is>
+          <t>University of Otago</t>
+        </is>
+      </c>
+      <c r="C260" s="5" t="inlineStr">
+        <is>
+          <t>West Visayas State University WVSU forges digital health alliance with New Zealand's University of Otago</t>
+        </is>
+      </c>
+      <c r="D260" s="5" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="E260" s="5" t="inlineStr">
+        <is>
+          <t>https://wvsu.edu.ph/wvsu-forges-digital-health-alliance-with-new-zealands-university-of-otago/</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="5" t="inlineStr">
+        <is>
+          <t>Sanford Health (Sanford World Clinic)</t>
+        </is>
+      </c>
+      <c r="B261" s="5" t="inlineStr">
+        <is>
+          <t>Omni Health (OmniHealth) primary care network</t>
+        </is>
+      </c>
+      <c r="C261" s="5" t="inlineStr">
+        <is>
+          <t>Sanford Health Sanford World Clinic New Zealand</t>
+        </is>
+      </c>
+      <c r="D261" s="5" t="inlineStr"/>
+      <c r="E261" s="5" t="inlineStr">
+        <is>
+          <t>https://www.sanfordhealth.org/initiatives/world-clinic/new-zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="5" t="inlineStr">
+        <is>
+          <t>Sanford Health (Sanford World Clinic)</t>
+        </is>
+      </c>
+      <c r="B262" s="5" t="inlineStr">
+        <is>
+          <t>Omni Health (OmniHealth) primary care network</t>
+        </is>
+      </c>
+      <c r="C262" s="5" t="inlineStr">
+        <is>
+          <t>Jodi Schwan Sanford World Clinic finds broader global reach despite pandemic</t>
+        </is>
+      </c>
+      <c r="D262" s="5" t="inlineStr">
+        <is>
+          <t>2021-05-17</t>
+        </is>
+      </c>
+      <c r="E262" s="5" t="inlineStr">
+        <is>
+          <t>https://siouxfalls.business/?p=89679</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="5" t="inlineStr">
+        <is>
+          <t>Sanford Health (Sanford World Clinic)</t>
+        </is>
+      </c>
+      <c r="B263" s="5" t="inlineStr">
+        <is>
+          <t>Omni Health (OmniHealth) primary care network</t>
+        </is>
+      </c>
+      <c r="C263" s="5" t="inlineStr">
+        <is>
+          <t>Sanford World Clinic Sanford World Clinic Partnering with Omni Health</t>
+        </is>
+      </c>
+      <c r="D263" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-06</t>
+        </is>
+      </c>
+      <c r="E263" s="5" t="inlineStr">
+        <is>
+          <t>https://employer.practicematch.com/employer/sanford-world-clinic/968142</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="5" t="inlineStr">
+        <is>
+          <t>Sanford Health (Sanford World Clinic)</t>
+        </is>
+      </c>
+      <c r="B264" s="5" t="inlineStr">
+        <is>
+          <t>Omni Health (OmniHealth) primary care network</t>
+        </is>
+      </c>
+      <c r="C264" s="5" t="inlineStr">
+        <is>
+          <t>New Zealand Doctor Big US health player buddies up with local network in new Auckland clinic</t>
+        </is>
+      </c>
+      <c r="D264" s="5" t="inlineStr"/>
+      <c r="E264" s="5" t="inlineStr">
+        <is>
+          <t>https://nzdoctor.co.nz/node/2668</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="5" t="inlineStr">
+        <is>
+          <t>Children's Cancer Institute and Sydney Children's Hospital, Randwick (Zero Childhood Cancer Program)</t>
+        </is>
+      </c>
+      <c r="B265" s="5" t="inlineStr">
+        <is>
+          <t>Starship Children's Hospital and Christchurch Hospital (Health New Zealand)</t>
+        </is>
+      </c>
+      <c r="C265" s="5" t="inlineStr">
+        <is>
+          <t>ANZCHOG ZERO2 opens in NZ</t>
+        </is>
+      </c>
+      <c r="D265" s="5" t="inlineStr">
+        <is>
+          <t>2024-08-19</t>
+        </is>
+      </c>
+      <c r="E265" s="5" t="inlineStr">
+        <is>
+          <t>https://anzchog.org/zero2-opens-in-nz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="5" t="inlineStr">
+        <is>
+          <t>Children's Cancer Institute and Sydney Children's Hospital, Randwick (Zero Childhood Cancer Program)</t>
+        </is>
+      </c>
+      <c r="B266" s="5" t="inlineStr">
+        <is>
+          <t>Starship Children's Hospital and Christchurch Hospital (Health New Zealand)</t>
+        </is>
+      </c>
+      <c r="C266" s="5" t="inlineStr">
+        <is>
+          <t>Children's Cancer Institute Zero Childhood Cancer</t>
+        </is>
+      </c>
+      <c r="D266" s="5" t="inlineStr"/>
+      <c r="E266" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ccia.org.au/personalised-medicine/zero-childhood-cancer</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="5" t="inlineStr">
+        <is>
+          <t>Children's Cancer Institute and Sydney Children's Hospital, Randwick (Zero Childhood Cancer Program)</t>
+        </is>
+      </c>
+      <c r="B267" s="5" t="inlineStr">
+        <is>
+          <t>Starship Children's Hospital and Christchurch Hospital (Health New Zealand)</t>
+        </is>
+      </c>
+      <c r="C267" s="5" t="inlineStr">
+        <is>
+          <t>ANZCHOG Precision Medicine for Every Child With Cancer (NCT05504772)</t>
+        </is>
+      </c>
+      <c r="D267" s="5" t="inlineStr">
+        <is>
+          <t>2024-07-17</t>
+        </is>
+      </c>
+      <c r="E267" s="5" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT05504772</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="5" t="inlineStr">
+        <is>
+          <t>Children's Hospital of Zhejiang University School of Medicine</t>
+        </is>
+      </c>
+      <c r="B268" s="5" t="inlineStr">
+        <is>
+          <t>NZ-China Non-Communicable Diseases Research Collaboration Centre (University of Otago)</t>
+        </is>
+      </c>
+      <c r="C268" s="5" t="inlineStr">
+        <is>
+          <t>NZ-China NCD Research Collaboration Centre NZ-China non-communicable disease research strengthened</t>
+        </is>
+      </c>
+      <c r="D268" s="5" t="inlineStr">
+        <is>
+          <t>2017-11-02</t>
+        </is>
+      </c>
+      <c r="E268" s="5" t="inlineStr">
+        <is>
+          <t>https://crcc.nz/crcc/?p=374</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="5" t="inlineStr">
+        <is>
+          <t>Children's Hospital of Zhejiang University School of Medicine</t>
+        </is>
+      </c>
+      <c r="B269" s="5" t="inlineStr">
+        <is>
+          <t>NZ-China Non-Communicable Diseases Research Collaboration Centre (University of Otago)</t>
+        </is>
+      </c>
+      <c r="C269" s="5" t="inlineStr">
+        <is>
+          <t>NZ-China NCD Research Collaboration Centre The 3rd NZ-China Non-Communicable Diseases Research Cooperation Forum deemed major success</t>
+        </is>
+      </c>
+      <c r="D269" s="5" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="E269" s="5" t="inlineStr">
+        <is>
+          <t>https://crcc.nz/crcc/?p=80</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="5" t="inlineStr">
+        <is>
+          <t>Fiji National University (College of Medicine, Nursing and Health Sciences)</t>
+        </is>
+      </c>
+      <c r="B270" s="5" t="inlineStr">
+        <is>
+          <t>University of Auckland</t>
+        </is>
+      </c>
+      <c r="C270" s="5" t="inlineStr">
+        <is>
+          <t>Fiji National University FNU formalises collaboration with the University of Auckland</t>
+        </is>
+      </c>
+      <c r="D270" s="5" t="inlineStr">
+        <is>
+          <t>2022-05-09</t>
+        </is>
+      </c>
+      <c r="E270" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fnu.ac.fj/?p=17198</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="5" t="inlineStr">
+        <is>
+          <t>Huashan Hospital (Fudan University)</t>
+        </is>
+      </c>
+      <c r="B271" s="5" t="inlineStr">
+        <is>
+          <t>NZ-China Non-Communicable Diseases Research Collaboration Centre (University of Otago)</t>
+        </is>
+      </c>
+      <c r="C271" s="5" t="inlineStr">
+        <is>
+          <t>NZ-China NCD Research Collaboration Centre NZ-China non-communicable disease research strengthened</t>
+        </is>
+      </c>
+      <c r="D271" s="5" t="inlineStr">
+        <is>
+          <t>2017-11-02</t>
+        </is>
+      </c>
+      <c r="E271" s="5" t="inlineStr">
+        <is>
+          <t>https://crcc.nz/crcc/?p=374</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="5" t="inlineStr">
+        <is>
+          <t>Huashan Hospital (Fudan University)</t>
+        </is>
+      </c>
+      <c r="B272" s="5" t="inlineStr">
+        <is>
+          <t>NZ-China Non-Communicable Diseases Research Collaboration Centre (University of Otago)</t>
+        </is>
+      </c>
+      <c r="C272" s="5" t="inlineStr">
+        <is>
+          <t>NZ-China NCD Research Collaboration Centre The 3rd NZ-China Non-Communicable Diseases Research Cooperation Forum deemed major success</t>
+        </is>
+      </c>
+      <c r="D272" s="5" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="E272" s="5" t="inlineStr">
+        <is>
+          <t>https://crcc.nz/crcc/?p=80</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="5" t="inlineStr">
+        <is>
+          <t>Shanghai Ninth People's Hospital (Shanghai Jiao Tong University School of Medicine)</t>
+        </is>
+      </c>
+      <c r="B273" s="5" t="inlineStr">
+        <is>
+          <t>University of Otago Faculty of Dentistry</t>
+        </is>
+      </c>
+      <c r="C273" s="5" t="inlineStr">
+        <is>
+          <t>Shanghai Jiao Tong University School of Medicine Shanghai Ninth People's Hospital and University of Otago Faculty of Dentistry in New Zealand Signed Memorandum of Understanding and Launched Joint Laboratory</t>
+        </is>
+      </c>
+      <c r="D273" s="5" t="inlineStr">
+        <is>
+          <t>2023-11-28</t>
+        </is>
+      </c>
+      <c r="E273" s="5" t="inlineStr">
+        <is>
+          <t>https://www.shsmu.edu.cn/english/info/1021/4710.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="5" t="inlineStr">
+        <is>
+          <t>Healthe Care Australia (then a subsidiary of Luye Medical Group)</t>
+        </is>
+      </c>
+      <c r="B274" s="5" t="inlineStr">
+        <is>
+          <t>Boulcott Hospital (Pulse Health NZ)</t>
+        </is>
+      </c>
+      <c r="C274" s="5" t="inlineStr">
+        <is>
+          <t>Commerce Commission Commission clears private hospitals merger subject to divestment</t>
+        </is>
+      </c>
+      <c r="D274" s="5" t="inlineStr">
+        <is>
+          <t>2021-11-17</t>
+        </is>
+      </c>
+      <c r="E274" s="5" t="inlineStr">
+        <is>
+          <t>https://comcom.govt.nz/news-and-media/media-releases/2021/commission-clears-private-hospitals-merger-subject-to-divestment</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="5" t="inlineStr">
+        <is>
+          <t>Healthe Care Australia (then a subsidiary of Luye Medical Group)</t>
+        </is>
+      </c>
+      <c r="B275" s="5" t="inlineStr">
+        <is>
+          <t>Boulcott Hospital (Pulse Health NZ)</t>
+        </is>
+      </c>
+      <c r="C275" s="5" t="inlineStr">
+        <is>
+          <t>Andrew Bevin Rangatira buys Boulcott Hospital operations for undisclosed sum</t>
+        </is>
+      </c>
+      <c r="D275" s="5" t="inlineStr">
+        <is>
+          <t>2022-03-02</t>
+        </is>
+      </c>
+      <c r="E275" s="5" t="inlineStr">
+        <is>
+          <t>https://nbr.co.nz/story/rangatira-buys-boulcott-hospital-operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Johns Hopkins Hospital)</t>
+        </is>
+      </c>
+      <c r="B276" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University (ABUAD)</t>
+        </is>
+      </c>
+      <c r="C276" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University ABUAD Tripartite agreement with John Hopkins University USA and Little by Little Foundation</t>
+        </is>
+      </c>
+      <c r="D276" s="5" t="inlineStr">
+        <is>
+          <t>2023-01-17</t>
+        </is>
+      </c>
+      <c r="E276" s="5" t="inlineStr">
+        <is>
+          <t>https://www.abuad.edu.ng/abuad-tripartite-agreement-with-john-hopkins-university-usa-and-little-by-little-foundation/</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Johns Hopkins Hospital)</t>
+        </is>
+      </c>
+      <c r="B277" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University (ABUAD)</t>
+        </is>
+      </c>
+      <c r="C277" s="5" t="inlineStr">
+        <is>
+          <t>ThisDay ABUAD, John Hopkins Partner to Boost Medical Training</t>
+        </is>
+      </c>
+      <c r="D277" s="5" t="inlineStr">
+        <is>
+          <t>2023-01-18</t>
+        </is>
+      </c>
+      <c r="E277" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2023/01/18/abuad-john-hopkins-partner-to-boost-medical-training/</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Johns Hopkins Hospital)</t>
+        </is>
+      </c>
+      <c r="B278" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University (ABUAD)</t>
+        </is>
+      </c>
+      <c r="C278" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University ABUAD Holds Seventh Induction Ceremony for Fresh Doctors</t>
+        </is>
+      </c>
+      <c r="D278" s="5" t="inlineStr">
+        <is>
+          <t>5 February 2025</t>
+        </is>
+      </c>
+      <c r="E278" s="5" t="inlineStr">
+        <is>
+          <t>https://vc.abuad.edu.ng/abuad-holds-seventh-induction-ceremony-for-fresh-doctors/</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic (Mayo Clinic Global Consulting)</t>
+        </is>
+      </c>
+      <c r="B279" s="5" t="inlineStr">
+        <is>
+          <t>Iwosan Investments Limited (Iwosan Lagoon Hospitals and Lagos Medipark Hospital)</t>
+        </is>
+      </c>
+      <c r="C279" s="5" t="inlineStr">
+        <is>
+          <t>The Sun Iwosan engages Mayo Clinic to advance high-quality patient-centered healthcare</t>
+        </is>
+      </c>
+      <c r="D279" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-17</t>
+        </is>
+      </c>
+      <c r="E279" s="5" t="inlineStr">
+        <is>
+          <t>https://thesun.ng/iwosan-engages-mayo-clinic-to-advance-high-quality-patient-centered-healthcare/</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic (Mayo Clinic Global Consulting)</t>
+        </is>
+      </c>
+      <c r="B280" s="5" t="inlineStr">
+        <is>
+          <t>Iwosan Investments Limited (Iwosan Lagoon Hospitals and Lagos Medipark Hospital)</t>
+        </is>
+      </c>
+      <c r="C280" s="5" t="inlineStr">
+        <is>
+          <t>BrandIconImage Iwosan Investments Limited Engages Mayo Clinic Global Consulting to Advance High-Quality Patient-Centered Healthcare in Nigeria</t>
+        </is>
+      </c>
+      <c r="D280" s="5" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="E280" s="5" t="inlineStr">
+        <is>
+          <t>https://www.brandiconimage.com/2025/04/iwosan-investments-limited-engages-mayo.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic (Mayo Clinic Global Consulting)</t>
+        </is>
+      </c>
+      <c r="B281" s="5" t="inlineStr">
+        <is>
+          <t>Iwosan Investments Limited (Iwosan Lagoon Hospitals and Lagos Medipark Hospital)</t>
+        </is>
+      </c>
+      <c r="C281" s="5" t="inlineStr">
+        <is>
+          <t>BusinessDay Iwosan engages Mayo Clinic to advance high quality patient centered healthcare in Nigeria</t>
+        </is>
+      </c>
+      <c r="D281" s="5" t="inlineStr">
+        <is>
+          <t>8 April 2025</t>
+        </is>
+      </c>
+      <c r="E281" s="5" t="inlineStr">
+        <is>
+          <t>https://businessday.ng/health/article/iwosan-engages-mayo-clinic-to-advance-high-quality-patient-centered-healthcare-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="B282" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH) and College of Medicine, University of Lagos</t>
+        </is>
+      </c>
+      <c r="C282" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center Global Cancer Research and Training Program 2025 Update</t>
+        </is>
+      </c>
+      <c r="D282" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E282" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mskcc.org/sites/default/files/node/118066/documents/gcrt_report_2026_6_01-29-98-44.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="B283" s="5" t="inlineStr">
+        <is>
+          <t>Obafemi Awolowo University Teaching Hospitals Complex (OAUTHC)</t>
+        </is>
+      </c>
+      <c r="C283" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center Global Cancer Research and Training Program 2025 Update</t>
+        </is>
+      </c>
+      <c r="D283" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E283" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mskcc.org/sites/default/files/node/118066/documents/gcrt_report_2026_6_01-29-98-44.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="B284" s="5" t="inlineStr">
+        <is>
+          <t>Obafemi Awolowo University Teaching Hospitals Complex (OAUTHC)</t>
+        </is>
+      </c>
+      <c r="C284" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center MSK's Global Cancer Research and Training (GCRT) Program</t>
+        </is>
+      </c>
+      <c r="D284" s="5" t="inlineStr"/>
+      <c r="E284" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mskcc.org/hcp-education-training/international/global-cancer-disparities-initiatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="B285" s="5" t="inlineStr">
+        <is>
+          <t>Abubakar Tafawa Balewa University Teaching Hospital (ATBUTH)</t>
+        </is>
+      </c>
+      <c r="C285" s="5" t="inlineStr">
+        <is>
+          <t>Leadership Bauchi Teaching Hospital Seeks Alliance To Strengthen Cancer Care</t>
+        </is>
+      </c>
+      <c r="D285" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-26</t>
+        </is>
+      </c>
+      <c r="E285" s="5" t="inlineStr">
+        <is>
+          <t>https://leadership.ng/bauchi-teaching-hospital-seeks-alliance-to-strengthen-cancer-care/</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="B286" s="5" t="inlineStr">
+        <is>
+          <t>The Dorcas Cancer Foundation (TDCF)</t>
+        </is>
+      </c>
+      <c r="C286" s="5" t="inlineStr">
+        <is>
+          <t>Sunday Ehigiator TDCF, St. Jude Global Alliance, Partner on Improving Pediatric Cancer Outcomes in Nigeria, Others</t>
+        </is>
+      </c>
+      <c r="D286" s="5" t="inlineStr">
+        <is>
+          <t>2024-12-17</t>
+        </is>
+      </c>
+      <c r="E286" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2024/12/17/tdcf-st-jude-global-alliance-partner-on-improving-pediatric-cancer-outcomes-in-nigeria-others/</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="B287" s="5" t="inlineStr">
+        <is>
+          <t>The Dorcas Cancer Foundation (TDCF)</t>
+        </is>
+      </c>
+      <c r="C287" s="5" t="inlineStr">
+        <is>
+          <t>BusinessDay TDCF admitted into St Jude Global Alliance to improve pediatric cancer outcomes in Nigeria</t>
+        </is>
+      </c>
+      <c r="D287" s="5" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="E287" s="5" t="inlineStr">
+        <is>
+          <t>https://businessday.ng/life/article/tdcf-admitted-into-st-jude-global-alliance-to-improve-pediatric-cancer-outcomes-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="5" t="inlineStr">
+        <is>
+          <t>University of Illinois Chicago (UIC School of Public Health)</t>
+        </is>
+      </c>
+      <c r="B288" s="5" t="inlineStr">
+        <is>
+          <t>Lagos State University (LASU)</t>
+        </is>
+      </c>
+      <c r="C288" s="5" t="inlineStr">
+        <is>
+          <t>UIC School of Public Health UIC and Lagos State University Sign Memorandum of Agreement</t>
+        </is>
+      </c>
+      <c r="D288" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E288" s="5" t="inlineStr">
+        <is>
+          <t>https://publichealth.uic.edu/news-stories/uic-and-lagos-state-university-sign-memorandum-of-agreement/</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine (Institute of Human Virology)</t>
+        </is>
+      </c>
+      <c r="B289" s="5" t="inlineStr">
+        <is>
+          <t>Institute of Human Virology Nigeria (IHVN)</t>
+        </is>
+      </c>
+      <c r="C289" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine University of Maryland Baltimore leadership helps IHV Nigeria launch campus in Abuja</t>
+        </is>
+      </c>
+      <c r="D289" s="5" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="E289" s="5" t="inlineStr">
+        <is>
+          <t>https://ihv.umaryland.edu/news/2023/university-of-maryland-baltimore-leadership-helps-ihv-nigeria-launch-state-of-the-art-campus-in-public-healthcare-treatment-training-and-research-in-nigeria.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine (Institute of Human Virology)</t>
+        </is>
+      </c>
+      <c r="B290" s="5" t="inlineStr">
+        <is>
+          <t>Institute of Human Virology Nigeria (IHVN)</t>
+        </is>
+      </c>
+      <c r="C290" s="5" t="inlineStr">
+        <is>
+          <t>US National Institutes of Health RePORTER: 5D43TW012280-05, Expanding the pool of Independent Investigators in Implementation Science (Institute of Human Virology Nigeria)</t>
+        </is>
+      </c>
+      <c r="D290" s="5" t="inlineStr">
+        <is>
+          <t>FY2026 (budget start 1 February 2026)</t>
+        </is>
+      </c>
+      <c r="E290" s="5" t="inlineStr">
+        <is>
+          <t>https://reporter.nih.gov/project-details/11251575</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="5" t="inlineStr">
+        <is>
+          <t>University of Miami (Sylvester Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="B291" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University Teaching Hospital (ABUTH)</t>
+        </is>
+      </c>
+      <c r="C291" s="5" t="inlineStr">
+        <is>
+          <t>ClinicalTrials.gov Study Evaluating Safety, Tolerability, and Metabolism of Niraparib (NCT06412120)</t>
+        </is>
+      </c>
+      <c r="D291" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E291" s="5" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT06412120</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="5" t="inlineStr">
+        <is>
+          <t>University of Miami (Sylvester Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="B292" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University Teaching Hospital (ABUTH)</t>
+        </is>
+      </c>
+      <c r="C292" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University ABUTH to begin clinical trials on ovarian cancer next year</t>
+        </is>
+      </c>
+      <c r="D292" s="5" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="E292" s="5" t="inlineStr">
+        <is>
+          <t>https://abu.edu.ng/abuth-to-begin-clinical-trials-on-ovarian-cancer-next-year/</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="5" t="inlineStr">
+        <is>
+          <t>University of Miami (Sylvester Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="B293" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University Teaching Hospital (ABUTH)</t>
+        </is>
+      </c>
+      <c r="C293" s="5" t="inlineStr">
+        <is>
+          <t>US National Library of Medicine NCT06412120: Niraparib as Maintenance Following Front-Line Treatment for Ovarian Cancer in Women of African Ancestry</t>
+        </is>
+      </c>
+      <c r="D293" s="5" t="inlineStr">
+        <is>
+          <t>5 August 2026</t>
+        </is>
+      </c>
+      <c r="E293" s="5" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT06412120</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="5" t="inlineStr">
+        <is>
+          <t>University of Virginia Health System</t>
+        </is>
+      </c>
+      <c r="B294" s="5" t="inlineStr">
+        <is>
+          <t>Federal Medical Centre Umuahia</t>
+        </is>
+      </c>
+      <c r="C294" s="5" t="inlineStr">
+        <is>
+          <t>UVA School of Medicine UVA Partners With Federal Medical Center in Nigeria to Elevate Global Kidney Care</t>
+        </is>
+      </c>
+      <c r="D294" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="E294" s="5" t="inlineStr">
+        <is>
+          <t>https://news.med.virginia.edu/community/uva-nigeria-elevating-global-kidney-care/</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="5" t="inlineStr">
+        <is>
+          <t>Vanderbilt University Medical Center (Vanderbilt Institute for Global Health)</t>
+        </is>
+      </c>
+      <c r="B295" s="5" t="inlineStr">
+        <is>
+          <t>Aminu Kano Teaching Hospital and Bayero University Kano</t>
+        </is>
+      </c>
+      <c r="C295" s="5" t="inlineStr">
+        <is>
+          <t>Fogarty International Center Vanderbilt-Nigeria Building Research Capacity in HIV and NCDs (V-BRCH)</t>
+        </is>
+      </c>
+      <c r="D295" s="5" t="inlineStr"/>
+      <c r="E295" s="5" t="inlineStr">
+        <is>
+          <t>https://fic.nih.gov/Grants/Search/Pages/hiv-research-training-d43tw011544.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="5" t="inlineStr">
+        <is>
+          <t>Vanderbilt University Medical Center (Vanderbilt Institute for Global Health)</t>
+        </is>
+      </c>
+      <c r="B296" s="5" t="inlineStr">
+        <is>
+          <t>Aminu Kano Teaching Hospital and Bayero University Kano</t>
+        </is>
+      </c>
+      <c r="C296" s="5" t="inlineStr">
+        <is>
+          <t>Vanderbilt Institute for Global Health V-BRCH</t>
+        </is>
+      </c>
+      <c r="D296" s="5" t="inlineStr"/>
+      <c r="E296" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vumc.org/global-health/v-brch</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="5" t="inlineStr">
+        <is>
+          <t>Vanderbilt University Medical Center (Vanderbilt Institute for Global Health)</t>
+        </is>
+      </c>
+      <c r="B297" s="5" t="inlineStr">
+        <is>
+          <t>Aminu Kano Teaching Hospital and Bayero University Kano</t>
+        </is>
+      </c>
+      <c r="C297" s="5" t="inlineStr">
+        <is>
+          <t>US National Institutes of Health RePORTER: 5D43TW011544-07, Vanderbilt-Nigeria Building Research Capacity in HIV and Non-communicable Diseases (V-BRCH)</t>
+        </is>
+      </c>
+      <c r="D297" s="5" t="inlineStr">
+        <is>
+          <t>FY2026 (budget start 1 January 2026)</t>
+        </is>
+      </c>
+      <c r="E297" s="5" t="inlineStr">
+        <is>
+          <t>https://reporter.nih.gov/project-details/11378551</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="5" t="inlineStr">
+        <is>
+          <t>Virginia Commonwealth University (VCU Massey Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="B298" s="5" t="inlineStr">
+        <is>
+          <t>National Hospital Abuja</t>
+        </is>
+      </c>
+      <c r="C298" s="5" t="inlineStr">
+        <is>
+          <t>Anthonia Obokoh National Hospital signs MoU with U.S. cancer center to boost research, clinical trials in Nigeria</t>
+        </is>
+      </c>
+      <c r="D298" s="5" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="E298" s="5" t="inlineStr">
+        <is>
+          <t>https://nairametrics.com/2025/07/01/national-hospital-signs-mou-with-u-s-cancer-center-to-boost-research-clinical-trials-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Group (owned at its 2021 launch by the TPG-managed Evercare Health Fund)</t>
+        </is>
+      </c>
+      <c r="B299" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Hospital Lekki</t>
+        </is>
+      </c>
+      <c r="C299" s="5" t="inlineStr">
+        <is>
+          <t>Esther Oluku Evercare, MedEI, Commence Advanced Cochlear Implant Surgery in Nigeria</t>
+        </is>
+      </c>
+      <c r="D299" s="5" t="inlineStr">
+        <is>
+          <t>2024-10-10</t>
+        </is>
+      </c>
+      <c r="E299" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2024/10/10/evercare-medei-commence-advanced-cochlear-implant-surgery-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Group (owned at its 2021 launch by the TPG-managed Evercare Health Fund)</t>
+        </is>
+      </c>
+      <c r="B300" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Hospital Lekki</t>
+        </is>
+      </c>
+      <c r="C300" s="5" t="inlineStr">
+        <is>
+          <t>TPG Evercare Group set to deliver accessible, quality healthcare in Nigeria</t>
+        </is>
+      </c>
+      <c r="D300" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E300" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tpg.com/news-and-insights/evercare-group-set-deliver-accessible-quality-healthcare-nigeria</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Group (owned at its 2021 launch by the TPG-managed Evercare Health Fund)</t>
+        </is>
+      </c>
+      <c r="B301" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Hospital Lekki</t>
+        </is>
+      </c>
+      <c r="C301" s="5" t="inlineStr">
+        <is>
+          <t>TPG Evercare Group set to deliver accessible, quality healthcare in Nigeria through a new world-class multispecialty hospital</t>
+        </is>
+      </c>
+      <c r="D301" s="5" t="inlineStr">
+        <is>
+          <t>26 February 2021</t>
+        </is>
+      </c>
+      <c r="E301" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tpg.com/news-and-insights/evercare-group-set-deliver-accessible-quality-healthcare-nigeria</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="5" t="inlineStr">
+        <is>
+          <t>King's College Hospital NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B302" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C302" s="5" t="inlineStr">
+        <is>
+          <t>Afreximbank King's College Hospital, London (KCH) affirmed as Clinical Partner</t>
+        </is>
+      </c>
+      <c r="D302" s="5" t="inlineStr">
+        <is>
+          <t>2021-06-03</t>
+        </is>
+      </c>
+      <c r="E302" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amce.net/?p=10738</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="5" t="inlineStr">
+        <is>
+          <t>King's College Hospital NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B303" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C303" s="5" t="inlineStr">
+        <is>
+          <t>Nnaemeka Onyekachi Afreximbank, BOI sign $75 million financing support for local manufacturers in Nigerian healthcare sector (reports AMCE commissioning)</t>
+        </is>
+      </c>
+      <c r="D303" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="E303" s="5" t="inlineStr">
+        <is>
+          <t>https://nairametrics.com/2025/06/05/afreximbank-boi-sign-75-million-financing-support-for-local-manufacturers-in-nigerian-healthcare-sector/</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="5" t="inlineStr">
+        <is>
+          <t>King's College Hospital NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B304" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C304" s="5" t="inlineStr">
+        <is>
+          <t>Brand Spur African Medical Centre Of Excellence Opens In Abuja As Nigeria Targets $2.2bn Health Sector Overhaul</t>
+        </is>
+      </c>
+      <c r="D304" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="E304" s="5" t="inlineStr">
+        <is>
+          <t>https://brandspurng.com/2026/09/19/african-medical-centre-of-excellence-opens-in-abuja-as-nigeria-targets-2-2bn-health-sector-overhaul/</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="5" t="inlineStr">
+        <is>
+          <t>King's College London</t>
+        </is>
+      </c>
+      <c r="B305" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C305" s="5" t="inlineStr">
+        <is>
+          <t>King's College London New partnership to deliver medical excellence in Nigeria</t>
+        </is>
+      </c>
+      <c r="D305" s="5" t="inlineStr">
+        <is>
+          <t>2023-11-28</t>
+        </is>
+      </c>
+      <c r="E305" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kcl.ac.uk/news/new-partnership-to-deliver-medical-excellence-in-nigeria</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="5" t="inlineStr">
+        <is>
+          <t>King's College London</t>
+        </is>
+      </c>
+      <c r="B306" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C306" s="5" t="inlineStr">
+        <is>
+          <t>Nnaemeka Onyekachi Afreximbank, BOI sign $75 million financing support for local manufacturers in Nigerian healthcare sector (reports KCL terms of agreement)</t>
+        </is>
+      </c>
+      <c r="D306" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="E306" s="5" t="inlineStr">
+        <is>
+          <t>https://nairametrics.com/2025/06/05/afreximbank-boi-sign-75-million-financing-support-for-local-manufacturers-in-nigerian-healthcare-sector/</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="5" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine</t>
+        </is>
+      </c>
+      <c r="B307" s="5" t="inlineStr">
+        <is>
+          <t>National Postgraduate Medical College of Nigeria (with Wellbeing Foundation Africa)</t>
+        </is>
+      </c>
+      <c r="C307" s="5" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine LSTM and Wellbeing Foundation Africa launch Advanced Training for Resident Doctors in Nigeria</t>
+        </is>
+      </c>
+      <c r="D307" s="5" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="E307" s="5" t="inlineStr">
+        <is>
+          <t>https://lstmed.ac.uk/news/liverpool-school-of-tropical-medicine-and-wellbeing-foundation-africa-launch-advanced-training-for-resident-doctors-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="5" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine</t>
+        </is>
+      </c>
+      <c r="B308" s="5" t="inlineStr">
+        <is>
+          <t>National Postgraduate Medical College of Nigeria (with Wellbeing Foundation Africa)</t>
+        </is>
+      </c>
+      <c r="C308" s="5" t="inlineStr">
+        <is>
+          <t>Wellbeing Foundation Africa AOSS Training Expands to Port Harcourt and Gombe</t>
+        </is>
+      </c>
+      <c r="D308" s="5" t="inlineStr">
+        <is>
+          <t>2025-05-22</t>
+        </is>
+      </c>
+      <c r="E308" s="5" t="inlineStr">
+        <is>
+          <t>https://wbfafrica.org/aoss-training-expands-to-port-harcourt-and-gombe-ghwp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="5" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine</t>
+        </is>
+      </c>
+      <c r="B309" s="5" t="inlineStr">
+        <is>
+          <t>National Postgraduate Medical College of Nigeria (with Wellbeing Foundation Africa)</t>
+        </is>
+      </c>
+      <c r="C309" s="5" t="inlineStr">
+        <is>
+          <t>Wellbeing Foundation Africa Liverpool School of Tropical Medicine, Wellbeing Foundation Africa, and Global Health Workforce Partnership</t>
+        </is>
+      </c>
+      <c r="D309" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-12</t>
+        </is>
+      </c>
+      <c r="E309" s="5" t="inlineStr">
+        <is>
+          <t>https://wbfafrica.org/liverpool-school-of-tropical-medicine-wellbeing-foundation-africa-and-global-health-workforce-partnership/</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="5" t="inlineStr">
+        <is>
+          <t>Manipal Hospitals</t>
+        </is>
+      </c>
+      <c r="B310" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University Multi-System Hospital</t>
+        </is>
+      </c>
+      <c r="C310" s="5" t="inlineStr">
+        <is>
+          <t>Folasade Akpan ABUAD multi-system hospital records 50 successful kidney transplants</t>
+        </is>
+      </c>
+      <c r="D310" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E310" s="5" t="inlineStr">
+        <is>
+          <t>https://nannews.ng/abuad-multi-system-hospital-records-50-successful-kidney-transplants/</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="5" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B311" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C311" s="5" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust The Christie International hosts African Medical Centre of Excellence visit</t>
+        </is>
+      </c>
+      <c r="D311" s="5" t="inlineStr">
+        <is>
+          <t>2024-10-25</t>
+        </is>
+      </c>
+      <c r="E311" s="5" t="inlineStr">
+        <is>
+          <t>https://christie.nhs.uk/about-us/news-at-the-christie/latest-news-stories/the-christie-international-hosts-african-medical-centre-of-excellence-visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="5" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B312" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C312" s="5" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust The Christie supporting a new African Medical Centre of Excellence project</t>
+        </is>
+      </c>
+      <c r="D312" s="5" t="inlineStr"/>
+      <c r="E312" s="5" t="inlineStr">
+        <is>
+          <t>https://christie.nhs.uk/about-us/about-the-christie/the-christie-international/partnerships-experience/the-christie-supporting-a-new-african-medical-centre-of-excellence-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="5" t="inlineStr">
+        <is>
+          <t>The Royal Marsden NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B313" s="5" t="inlineStr">
+        <is>
+          <t>Marcelle Ruth Cancer Centre &amp; Specialist Hospital</t>
+        </is>
+      </c>
+      <c r="C313" s="5" t="inlineStr">
+        <is>
+          <t>BusinessDay Marcelle Ruth Cancer Centre partners UK's Royal Marsden to improve healthcare delivery in West Africa</t>
+        </is>
+      </c>
+      <c r="D313" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E313" s="5" t="inlineStr">
+        <is>
+          <t>https://businessday.ng/news/article/marcelle-ruth-cancer-centre-royal-marsden-partner-to-elevate-west-africas-oncology-care/</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="5" t="inlineStr">
+        <is>
+          <t>University of Birmingham</t>
+        </is>
+      </c>
+      <c r="B314" s="5" t="inlineStr">
+        <is>
+          <t>University of Lagos (with Lagos University Teaching Hospital)</t>
+        </is>
+      </c>
+      <c r="C314" s="5" t="inlineStr">
+        <is>
+          <t>Adesina Wahab UNILAG, University of Birmingham sign MoU on Transnational Education Engagement</t>
+        </is>
+      </c>
+      <c r="D314" s="5" t="inlineStr">
+        <is>
+          <t>29 January 2026</t>
+        </is>
+      </c>
+      <c r="E314" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vanguardngr.com/2026/01/unilag-university-of-birmingham-sign-mou-on-transnational-education-engagement/</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="5" t="inlineStr">
+        <is>
+          <t>University of Glasgow</t>
+        </is>
+      </c>
+      <c r="B315" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University</t>
+        </is>
+      </c>
+      <c r="C315" s="5" t="inlineStr">
+        <is>
+          <t>University of Glasgow School of Infection &amp; Immunity's Professor Harry de-Koning helps facilitate UofG-ABU MoU</t>
+        </is>
+      </c>
+      <c r="D315" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="E315" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gla.ac.uk/schools/infectionimmunity/newsevents/headline_1265451_en.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine</t>
+        </is>
+      </c>
+      <c r="B316" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH)</t>
+        </is>
+      </c>
+      <c r="C316" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital Maryland LUTH</t>
+        </is>
+      </c>
+      <c r="D316" s="5" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="E316" s="5" t="inlineStr">
+        <is>
+          <t>https://luth.gov.ng/news/maryland-luth</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine</t>
+        </is>
+      </c>
+      <c r="B317" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH)</t>
+        </is>
+      </c>
+      <c r="C317" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital University of Maryland School of Medicine Collaborates with Lagos University Teaching Hospital on Non-Communicable Diseases</t>
+        </is>
+      </c>
+      <c r="D317" s="5" t="inlineStr">
+        <is>
+          <t>August 2024</t>
+        </is>
+      </c>
+      <c r="E317" s="5" t="inlineStr">
+        <is>
+          <t>https://luth.gov.ng/news/maryland-luth</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine</t>
+        </is>
+      </c>
+      <c r="B318" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH)</t>
+        </is>
+      </c>
+      <c r="C318" s="5" t="inlineStr">
+        <is>
+          <t>IHV Nigeria University of Maryland Dean of Medicine Visits LUTH</t>
+        </is>
+      </c>
+      <c r="D318" s="5" t="inlineStr">
+        <is>
+          <t>August 2024</t>
+        </is>
+      </c>
+      <c r="E318" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ihvnigeria.org/university-of-maryland-dean-of-medicine-visits-luth/</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="5" t="inlineStr">
+        <is>
+          <t>University of Virginia Health System</t>
+        </is>
+      </c>
+      <c r="B319" s="5" t="inlineStr">
+        <is>
+          <t>Federal Medical Centre Owo</t>
+        </is>
+      </c>
+      <c r="C319" s="5" t="inlineStr">
+        <is>
+          <t>UVA School of Medicine UVA Department of Nephrology Partners With Nigerian Federal Medical Center</t>
+        </is>
+      </c>
+      <c r="D319" s="5" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="E319" s="5" t="inlineStr">
+        <is>
+          <t>https://news.med.virginia.edu/community/uva-department-of-nephrology-partners-with-nigerian-federal-medical-center/</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="5" t="inlineStr">
+        <is>
+          <t>Yale School of Medicine (Department of Psychiatry)</t>
+        </is>
+      </c>
+      <c r="B320" s="5" t="inlineStr">
+        <is>
+          <t>Imo State University Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="C320" s="5" t="inlineStr">
+        <is>
+          <t>Nigeria Health Watch Making Happiness Local: How a Project is Improving Access to Mental Healthcare in Imo State</t>
+        </is>
+      </c>
+      <c r="D320" s="5" t="inlineStr">
+        <is>
+          <t>2023-09-06</t>
+        </is>
+      </c>
+      <c r="E320" s="5" t="inlineStr">
+        <is>
+          <t>https://nigeriahealthwatch.com/articles/torchlight/making-happiness-local-how-a-project-is-improving-access-to-mental-healthcare-in-imo-state/</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="5" t="inlineStr">
+        <is>
+          <t>Yale School of Medicine (Department of Psychiatry)</t>
+        </is>
+      </c>
+      <c r="B321" s="5" t="inlineStr">
+        <is>
+          <t>Imo State University Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="C321" s="5" t="inlineStr">
+        <is>
+          <t>Yale School of Medicine The HAPPINESS Project</t>
+        </is>
+      </c>
+      <c r="D321" s="5" t="inlineStr"/>
+      <c r="E321" s="5" t="inlineStr">
+        <is>
+          <t>https://medicine.yale.edu/psychiatry/education/programs-and-initiatives/happiness</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B322" s="5" t="inlineStr">
+        <is>
+          <t>Duchess International Hospital (Reddington Hospital Group)</t>
+        </is>
+      </c>
+      <c r="C322" s="5" t="inlineStr">
+        <is>
+          <t>ThisDay Duchess International Hospital Has Put Lagos on World Healthcare Map, Says US Consul General</t>
+        </is>
+      </c>
+      <c r="D322" s="5" t="inlineStr">
+        <is>
+          <t>11 November 2021</t>
+        </is>
+      </c>
+      <c r="E322" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/index.php/2021/11/11/duchess-international-hospital-has-put-lagos-on-world-healthcare-map-says-us-consul-general/</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B323" s="5" t="inlineStr">
+        <is>
+          <t>Duchess International Hospital (Reddington Hospital Group)</t>
+        </is>
+      </c>
+      <c r="C323" s="5" t="inlineStr">
+        <is>
+          <t>Appolonia Adeyemi Duchess International Hospital debuts in Lagos, builds capacity</t>
+        </is>
+      </c>
+      <c r="D323" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E323" s="5" t="inlineStr">
+        <is>
+          <t>https://newtelegraphng.com/?p=192437</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B324" s="5" t="inlineStr">
+        <is>
+          <t>State House Clinic</t>
+        </is>
+      </c>
+      <c r="C324" s="5" t="inlineStr">
+        <is>
+          <t>Blueprint State House Clinic, Indian hospital collaborate to assist heart, kidney, cancer patients</t>
+        </is>
+      </c>
+      <c r="D324" s="5" t="inlineStr">
+        <is>
+          <t>2022-07-29</t>
+        </is>
+      </c>
+      <c r="E324" s="5" t="inlineStr">
+        <is>
+          <t>https://blueprint.ng/state-house-clinic-indian-hospital-collaborate-to-assist-heart-kidney-cancer-patients/</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B325" s="5" t="inlineStr">
+        <is>
+          <t>State House Clinic</t>
+        </is>
+      </c>
+      <c r="C325" s="5" t="inlineStr">
+        <is>
+          <t>ThisDay Medical Tourism: Indian Hospital to Train Nigerian Doctors on Cancer Treatment</t>
+        </is>
+      </c>
+      <c r="D325" s="5" t="inlineStr">
+        <is>
+          <t>2024-03-05</t>
+        </is>
+      </c>
+      <c r="E325" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2024/03/05/medical-tourism-indian-hospital-to-train-nigerian-doctors-on-cancer-treatment/</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Hospitals Group</t>
+        </is>
+      </c>
+      <c r="B326" s="5" t="inlineStr">
+        <is>
+          <t>Kasi Healthcare</t>
+        </is>
+      </c>
+      <c r="C326" s="5" t="inlineStr">
+        <is>
+          <t>Temitayo Ayetoto-Oladehinde Nigeria partners Turkey to tap $8.5trn healthcare market</t>
+        </is>
+      </c>
+      <c r="D326" s="5" t="inlineStr">
+        <is>
+          <t>2024-09-27</t>
+        </is>
+      </c>
+      <c r="E326" s="5" t="inlineStr">
+        <is>
+          <t>https://businessday.ng/news/article/nigeria-partners-turkey-to-tap-8-5trn-healthcare-market/</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="5" t="inlineStr">
+        <is>
+          <t>Peking University People's Hospital (named variously in press as People's University Hospital, Beijing)</t>
+        </is>
+      </c>
+      <c r="B327" s="5" t="inlineStr">
+        <is>
+          <t>University of Abuja Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="C327" s="5" t="inlineStr">
+        <is>
+          <t>Within Nigeria Nigeria signs letter of intent with China to improve health sector</t>
+        </is>
+      </c>
+      <c r="D327" s="5" t="inlineStr">
+        <is>
+          <t>2022-08-20</t>
+        </is>
+      </c>
+      <c r="E327" s="5" t="inlineStr">
+        <is>
+          <t>https://www.withinnigeria.com/broadnews/2022/08/20/nigeria-signs-letter-of-intent-with-china-to-improve-health-sector/</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="5" t="inlineStr">
+        <is>
+          <t>Peking University People's Hospital (named variously in press as People's University Hospital, Beijing)</t>
+        </is>
+      </c>
+      <c r="B328" s="5" t="inlineStr">
+        <is>
+          <t>University of Abuja Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="C328" s="5" t="inlineStr">
+        <is>
+          <t>University of Abuja Teaching Hospital Nigeria, China signs letter of intent to improve health sector</t>
+        </is>
+      </c>
+      <c r="D328" s="5" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="E328" s="5" t="inlineStr">
+        <is>
+          <t>https://uathospital.ng/nigeria-china-signs-letter-of-intent-to-improve-health-sector/</t>
         </is>
       </c>
     </row>
@@ -14703,6 +19460,90 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E242" r:id="rId241"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E243" r:id="rId242"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E300" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E301" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E302" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E303" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E304" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E305" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E306" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E307" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E308" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E309" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E310" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E311" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E312" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E313" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E314" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E315" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E316" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E317" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E318" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E319" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E320" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E321" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E322" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E323" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E324" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E325" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E326" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E327" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E328" r:id="rId327"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>